<commit_message>
Shop-built side truss: 60x60x2 bottom chord, apex bearing plate, node B axonometry and assembly sequence
- side truss (chord, two diagonals, 370x80x8 bearing plate) is fully shop-welded;
  middle frame stubs land on the plate and are welded on site
- model: apex_z option and shop truss geometry; all checks pass (max u 0.96)
- nodes drawing: new node B views + axonometry, full truss elevation, node C,
  shop/site assembly sequence, weld checks; node A gussets fitted on site
- drawings for the contractor no longer show any prices
- reply to the contractor's questions, decisions log updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X6AG5Fdm1RBCCrsAG1aTU6
</commit_message>
<xml_diff>
--- a/output/smeta_optimized.xlsx
+++ b/output/smeta_optimized.xlsx
@@ -480,7 +480,7 @@
         <v>75812</v>
       </c>
       <c r="C2" t="n">
-        <v>44600</v>
+        <v>45525</v>
       </c>
       <c r="D2">
         <f>C2-B2</f>
@@ -502,7 +502,7 @@
         <v>1647</v>
       </c>
       <c r="C3" t="n">
-        <v>1453</v>
+        <v>1658</v>
       </c>
       <c r="D3">
         <f>C3-B3</f>
@@ -678,7 +678,7 @@
         <v>5500</v>
       </c>
       <c r="C11" t="n">
-        <v>3813</v>
+        <v>3911</v>
       </c>
       <c r="D11">
         <f>C11-B11</f>
@@ -700,7 +700,7 @@
         <v>6600</v>
       </c>
       <c r="C12" t="n">
-        <v>3792</v>
+        <v>3862</v>
       </c>
       <c r="D12">
         <f>C12-B12</f>
@@ -810,7 +810,7 @@
         <v>24000</v>
       </c>
       <c r="C17" t="n">
-        <v>13799</v>
+        <v>13913</v>
       </c>
       <c r="D17">
         <f>C17-B17</f>
@@ -832,7 +832,7 @@
         <v>7000</v>
       </c>
       <c r="C18" t="n">
-        <v>4853</v>
+        <v>4977</v>
       </c>
       <c r="D18">
         <f>C18-B18</f>
@@ -854,7 +854,7 @@
         <v>15000</v>
       </c>
       <c r="C19" t="n">
-        <v>8625</v>
+        <v>8695</v>
       </c>
       <c r="D19">
         <f>C19-B19</f>
@@ -920,7 +920,7 @@
         <v>7000</v>
       </c>
       <c r="C22" t="n">
-        <v>4025</v>
+        <v>4058</v>
       </c>
       <c r="D22">
         <f>C22-B22</f>
@@ -961,7 +961,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Масса металла: было 1226 кг, стало 745 кг; площадь окраски 57.6 → 39.9 м²; швы 37.6 → 21.6 м; деталей 84 → 52.</t>
+          <t>Масса металла: было 1226 кг, стало 763 кг; площадь окраски 57.6 → 40.9 м²; швы 37.6 → 22.0 м; деталей 84 → 52.</t>
         </is>
       </c>
     </row>
@@ -1033,23 +1033,23 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы, Обрешётка</t>
+          <t>Обрешётка</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>162.83</v>
+        <v>153.63</v>
       </c>
       <c r="D2" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E2" t="n">
-        <v>324.3</v>
+        <v>306</v>
       </c>
       <c r="F2" t="n">
         <v>127</v>
       </c>
       <c r="G2" t="n">
-        <v>20680</v>
+        <v>19511</v>
       </c>
     </row>
     <row r="3">
@@ -1114,23 +1114,23 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Затяжки, Раскосы боковой фермы</t>
+          <t>Затяжки, Нижний пояс боковой фермы, Раскосы боковой фермы</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>26.27</v>
+        <v>35.41</v>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E5" t="n">
-        <v>93.59999999999999</v>
+        <v>126.1</v>
       </c>
       <c r="F5" t="n">
         <v>226</v>
       </c>
       <c r="G5" t="n">
-        <v>5937</v>
+        <v>8003</v>
       </c>
     </row>
     <row r="6">
@@ -1172,19 +1172,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.21</v>
+        <v>0.3</v>
       </c>
       <c r="D7" t="n">
         <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
       <c r="F7" t="n">
         <v>315</v>
       </c>
       <c r="G7" t="n">
-        <v>65</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8">
@@ -1209,7 +1209,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Пластины (фасонки, крышки колонн): 26.4 кг × 55 грн/кг</t>
+          <t>Пластины (фасонки, крышки колонн): 30.1 кг × 55 грн/кг</t>
         </is>
       </c>
     </row>
@@ -1565,17 +1565,17 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2.383</v>
+        <v>2.403</v>
       </c>
       <c r="D13" t="n">
         <v>4</v>
       </c>
       <c r="E13" t="n">
-        <v>33.9</v>
+        <v>34.2</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>оба торца — вертикальные резы (69.7° к оси)</t>
+          <t>оба торца — горизонтальные резы под 20.7° к оси (рез по грани 170 мм): низ — на пояс, верх — под столик</t>
         </is>
       </c>
     </row>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1597,11 +1597,11 @@
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>18.1</v>
+        <v>32.3</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>оба торца — прямые, между гранями колонн</t>
+          <t>оба торца — прямые; по фактическому расстоянию между гранями колонн</t>
         </is>
       </c>
     </row>
@@ -1627,7 +1627,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>низ — прямой (+ заглушка), верх — под 12°</t>
+          <t>низ — прямой (встаёт на столик фермы), верх — под 12°</t>
         </is>
       </c>
     </row>
@@ -1817,16 +1817,16 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.357 + 2.383 + 2.383</t>
+          <t>5.357 + 4.540</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Затяжка крайней рамы; Раскос боковой фермы</t>
+          <t>Затяжка крайней рамы; Нижний пояс боковой фермы</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1.868</v>
+        <v>2.097</v>
       </c>
     </row>
     <row r="8">
@@ -1837,52 +1837,52 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>3 (6 м)</t>
+          <t>3 (12 м)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2.383 + 2.383</t>
+          <t>4.540 + 2.403 + 2.403 + 2.403</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы</t>
+          <t>Нижний пояс боковой фермы; Раскос боковой фермы</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1.228</v>
+        <v>0.239</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>□20×20×2</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1 (12 м)</t>
+          <t>4 (6 м)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.598 + 0.598 + 0.598</t>
+          <t>2.403</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Подвеска у конька; Подкос фермы</t>
+          <t>Раскос боковой фермы</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>4.479</v>
+        <v>3.594</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1892,16 +1892,16 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>5.780 + 5.780</t>
+          <t>0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.598 + 0.598 + 0.598</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (край → рама 3)</t>
+          <t>Подвеска у конька; Подкос фермы</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.434</v>
+        <v>4.479</v>
       </c>
     </row>
     <row r="11">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2 (12 м)</t>
+          <t>1 (12 м)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>3 (12 м)</t>
+          <t>2 (12 м)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1962,7 +1962,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>4 (12 м)</t>
+          <t>3 (12 м)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>5 (12 м)</t>
+          <t>4 (12 м)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2012,7 +2012,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>6 (12 м)</t>
+          <t>5 (12 м)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>7 (12 м)</t>
+          <t>6 (12 м)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>8 (12 м)</t>
+          <t>7 (12 м)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>9 (12 м)</t>
+          <t>8 (12 м)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10 (12 м)</t>
+          <t>9 (12 м)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11 (12 м)</t>
+          <t>10 (12 м)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2162,21 +2162,21 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>12 (12 м)</t>
+          <t>11 (12 м)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>4.540 + 4.540 + 1.200 + 1.200</t>
+          <t>5.780 + 5.780</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы; Обрешётина, часть 2 (рама 3 → край)</t>
+          <t>Обрешётина, часть 1 (край → рама 3)</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.508</v>
+        <v>0.434</v>
       </c>
     </row>
     <row r="22">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>13 (12 м)</t>
+          <t>12 (12 м)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2212,7 +2212,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>14 (12 м)</t>
+          <t>13 (12 м)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2237,12 +2237,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>15 (6 м)</t>
+          <t>14 (6 м)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1.200 + 1.200</t>
+          <t>1.200 + 1.200 + 1.200 + 1.200</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2251,7 +2251,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>3.594</v>
+        <v>1.188</v>
       </c>
     </row>
     <row r="25">
@@ -2687,7 +2687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2739,7 +2739,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Фасонка</t>
+          <t>Фасонка узла А</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2751,174 +2751,205 @@
         <v>5</v>
       </c>
       <c r="D2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E2" t="n">
-        <v>23.08</v>
+        <v>15.39</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>узлы А (4 × 2) и Б (2 × 2)</t>
+          <t>узлы А (4 × 2), ставятся на объекте</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>полоса 250 мм из листа t=5: 6 пар «валетом» по 392 мм → 250 × 2352</t>
+          <t>полоса 250 мм из листа t=5: 4 пары «валетом» по 392 мм → 250 × 1568</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Опорная пластина под стропило</t>
+          <t>Фасонка узла Б</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>140 × 60</t>
+          <t>трапеция 230 × 164 / 213</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>2.37</v>
+        <v>6.79</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>верх колонн и стоек-вставок</t>
+          <t>узлы Б (2 × 2), в цеху на средней раме</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>полоса 60×6: 6 × 140 = 840 мм</t>
+          <t>полоса 230 мм из листа t=5: 2 пары «валетом» по 377 мм → 230 × 754</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Заглушка низа колонны</t>
+          <t>Опорный столик боковой фермы</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>110 × 70</t>
+          <t>370 × 80</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>0.97</v>
+        <v>3.72</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>низ колонн в лунке</t>
+          <t>вершина боковой фермы</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>лист t=4: 4 шт → 220 × 140</t>
+          <t>полоса 80×8: 2 × 370 = 740 мм</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Заглушка низа стойки-вставки</t>
+          <t>Опорная пластина под стропило</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>60 × 60</t>
+          <t>140 × 60</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E5" t="n">
-        <v>0.17</v>
+        <v>2.37</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>узел Б</t>
+          <t>верх колонн и стоек-вставок</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>полоса 60×3: 2 × 60 = 120 мм</t>
+          <t>полоса 60×6: 6 × 140 = 840 мм</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Заглушка торца стропила в свесе</t>
+          <t>Заглушка низа колонны</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>100 × 60</t>
+          <t>110 × 70</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>0.57</v>
+        <v>0.97</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>концы стропил у карниза</t>
+          <t>низ колонн в лунке</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>лист t=2 (или пластиковые заглушки 100×60)</t>
+          <t>лист t=4: 4 шт → 220 × 140</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Заглушка торца стропила в свесе</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>100 × 60</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>концы стропил у карниза</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>лист t=2 (или пластиковые заглушки 100×60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Заглушка торца обрешётины</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>35 × 35</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D8" t="n">
         <v>44</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E8" t="n">
         <v>0</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>торцы обрешётин на кромках кровли</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>пластиковые заглушки 35×35</t>
         </is>
@@ -2996,20 +3027,20 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>24.06</v>
+        <v>24.1</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>2.5</v>
+        <v>2.511</v>
       </c>
       <c r="F2" t="n">
-        <v>0.849</v>
+        <v>0.857</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>гибкость [D+S+0.9W+y]</t>
+          <t>гибкость [D+S]</t>
         </is>
       </c>
     </row>
@@ -3025,13 +3056,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.11</v>
+        <v>28.09</v>
       </c>
       <c r="D3" t="n">
         <v>0.8</v>
       </c>
       <c r="E3" t="n">
-        <v>4.063</v>
+        <v>4.073</v>
       </c>
       <c r="F3" t="n">
         <v>0.959</v>
@@ -3054,13 +3085,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.54</v>
+        <v>0.57</v>
       </c>
       <c r="D4" t="n">
-        <v>26.38</v>
+        <v>26.35</v>
       </c>
       <c r="E4" t="n">
-        <v>0.365</v>
+        <v>0.367</v>
       </c>
       <c r="F4" t="n">
         <v>0.772</v>
@@ -3141,10 +3172,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.83</v>
+        <v>0.88</v>
       </c>
       <c r="D7" t="n">
-        <v>1.98</v>
+        <v>2.1</v>
       </c>
       <c r="E7" t="n">
         <v>0.438</v>
@@ -3170,13 +3201,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19.95</v>
+        <v>20.87</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>0.18</v>
+        <v>0.166</v>
       </c>
       <c r="F8" t="n">
         <v>0.643</v>
@@ -3195,24 +3226,24 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>16.68</v>
+        <v>17.85</v>
       </c>
       <c r="E9" t="n">
-        <v>0.045</v>
+        <v>0.12</v>
       </c>
       <c r="F9" t="n">
-        <v>0.864</v>
+        <v>0.643</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>гибкость раст. [D+S]</t>
+          <t>стенка c/t изг. [D+S]</t>
         </is>
       </c>
     </row>
@@ -3228,20 +3259,20 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>13.67</v>
+        <v>13.97</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>1.946</v>
+        <v>1.95</v>
       </c>
       <c r="F10" t="n">
-        <v>0.836</v>
+        <v>0.83</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>устойчивость [D+S+0.9W+y]</t>
+          <t>устойчивость [D+S]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bars: 6 m only below 70x70 (contractor data); lath 6.98 m in two parts with a full-strength insert splice in the span; splice detail, cutting plan, reply and explanation PDF updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X6AG5Fdm1RBCCrsAG1aTU6
</commit_message>
<xml_diff>
--- a/output/smeta_optimized.xlsx
+++ b/output/smeta_optimized.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Сравнение" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Ведомость металла" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Детали" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Раскрой (хлысты 6 и 12 м)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Раскрой на хлысты" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Металлочерепица" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Пластины" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Проверки" sheetId="7" state="visible" r:id="rId7"/>
@@ -480,7 +480,7 @@
         <v>75812</v>
       </c>
       <c r="C2" t="n">
-        <v>45525</v>
+        <v>45534</v>
       </c>
       <c r="D2">
         <f>C2-B2</f>
@@ -700,7 +700,7 @@
         <v>6600</v>
       </c>
       <c r="C12" t="n">
-        <v>3862</v>
+        <v>4377</v>
       </c>
       <c r="D12">
         <f>C12-B12</f>
@@ -810,7 +810,7 @@
         <v>24000</v>
       </c>
       <c r="C17" t="n">
-        <v>13913</v>
+        <v>17121</v>
       </c>
       <c r="D17">
         <f>C17-B17</f>
@@ -854,7 +854,7 @@
         <v>15000</v>
       </c>
       <c r="C19" t="n">
-        <v>8695</v>
+        <v>10700</v>
       </c>
       <c r="D19">
         <f>C19-B19</f>
@@ -920,7 +920,7 @@
         <v>7000</v>
       </c>
       <c r="C22" t="n">
-        <v>4058</v>
+        <v>4993</v>
       </c>
       <c r="D22">
         <f>C22-B22</f>
@@ -961,7 +961,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Масса металла: было 1226 кг, стало 763 кг; площадь окраски 57.6 → 40.9 м²; швы 37.6 → 22.0 м; деталей 84 → 52.</t>
+          <t>Масса металла: было 1226 кг, стало 763 кг; площадь окраски 57.6 → 40.9 м²; швы 37.6 → 24.9 м; деталей 84 → 74.</t>
         </is>
       </c>
     </row>
@@ -1037,19 +1037,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>153.63</v>
+        <v>153.69</v>
       </c>
       <c r="D2" t="n">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="E2" t="n">
-        <v>306</v>
+        <v>306.1</v>
       </c>
       <c r="F2" t="n">
         <v>127</v>
       </c>
       <c r="G2" t="n">
-        <v>19511</v>
+        <v>19519</v>
       </c>
     </row>
     <row r="3">
@@ -1224,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1530,102 +1530,154 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Обрешётина цельная</t>
+          <t>Вкладыш стыка обрешётины</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□30×30×2</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6.98</v>
+        <v>0.1</v>
       </c>
       <c r="D12" t="n">
         <v>22</v>
       </c>
       <c r="E12" t="n">
-        <v>305.8</v>
+        <v>3.7</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>торцы прямые; из хлыста 12 м, без стыка</t>
+          <t>отрезок трубы внутрь стыка, по 50 мм в каждую часть</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2.403</v>
+        <v>5.49</v>
       </c>
       <c r="D13" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="E13" t="n">
-        <v>34.2</v>
+        <v>240.5</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>оба торца — горизонтальные резы под 20.7° к оси (рез по грани 170 мм): низ — на пояс, верх — под столик</t>
+          <t>торцы прямые; стык с частью 2 — в пролёте, в 290 мм от стропила рамы 3 (на вкладыше, см. узлы)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4.54</v>
+        <v>1.49</v>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="E14" t="n">
-        <v>32.3</v>
+        <v>65.3</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>оба торца — прямые; по фактическому расстоянию между гранями колонн</t>
+          <t>торцы прямые</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Раскос боковой фермы</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>□60×60×2</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2.403</v>
+      </c>
+      <c r="D15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>оба торца — горизонтальные резы под 20.7° к оси (рез по грани 170 мм): низ — на пояс, верх — под столик</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Нижний пояс боковой фермы</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>□60×60×2</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>оба торца — прямые; по фактическому расстоянию между гранями колонн</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Стойка-вставка</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>□60×60×3</t>
         </is>
       </c>
-      <c r="C15" t="n">
+      <c r="C17" t="n">
         <v>0.113</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D17" t="n">
         <v>2</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E17" t="n">
         <v>1.2</v>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>низ — прямой (встаёт на столик фермы), верх — под 12°</t>
         </is>
@@ -1642,7 +1694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1687,21 +1739,21 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1 (12 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>4.013 + 3.993 + 3.833</t>
+          <t>4.013</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Колонна Л3; Колонна П1; Колонна П3</t>
+          <t>Колонна П3</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.152</v>
+        <v>1.984</v>
       </c>
     </row>
     <row r="3">
@@ -1717,147 +1769,147 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>3.803</t>
+          <t>3.993</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Колонна Л1</t>
+          <t>Колонна Л3</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2.194</v>
+        <v>2.004</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>□100×60×3</t>
+          <t>□100×60×4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1 (12 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.710 + 3.710 + 3.710</t>
+          <t>3.833</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Стропило длинное (свес 0.90)</t>
+          <t>Колонна П1</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.861</v>
+        <v>2.164</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>□100×60×3</t>
+          <t>□100×60×4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2 (12 м)</t>
+          <t>4 (6 м)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.199 + 3.199 + 3.199</t>
+          <t>3.803</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Стропило короткое (свес 0.40)</t>
+          <t>Колонна Л1</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2.394</v>
+        <v>2.194</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□100×60×3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1 (12 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.397 + 5.357</t>
+          <t>3.710</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Затяжка крайней рамы; Затяжка средней рамы</t>
+          <t>Стропило длинное (свес 0.90)</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1.24</v>
+        <v>2.287</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□100×60×3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2 (12 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.357 + 4.540</t>
+          <t>3.710</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Затяжка крайней рамы; Нижний пояс боковой фермы</t>
+          <t>Стропило длинное (свес 0.90)</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>2.097</v>
+        <v>2.287</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□100×60×3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>3 (12 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>4.540 + 2.403 + 2.403 + 2.403</t>
+          <t>3.710</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы; Раскос боковой фермы</t>
+          <t>Стропило длинное (свес 0.90)</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.239</v>
+        <v>2.287</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□100×60×3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1867,316 +1919,316 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2.403</t>
+          <t>3.199</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы</t>
+          <t>Стропило короткое (свес 0.40)</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3.594</v>
+        <v>2.798</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>□20×20×2</t>
+          <t>□100×60×3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1 (12 м)</t>
+          <t>5 (6 м)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.598 + 0.598 + 0.598</t>
+          <t>3.199</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Подвеска у конька; Подкос фермы</t>
+          <t>Стропило короткое (свес 0.40)</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>4.479</v>
+        <v>2.798</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□100×60×3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1 (12 м)</t>
+          <t>6 (6 м)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>5.780 + 5.780</t>
+          <t>3.199</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (край → рама 3)</t>
+          <t>Стропило короткое (свес 0.40)</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.434</v>
+        <v>2.798</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2 (12 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>5.780 + 5.780</t>
+          <t>5.397</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (край → рама 3)</t>
+          <t>Затяжка средней рамы</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.434</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>3 (12 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>5.780 + 5.780</t>
+          <t>5.357</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (край → рама 3)</t>
+          <t>Затяжка крайней рамы</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.434</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>4 (12 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.780 + 5.780</t>
+          <t>5.357</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (край → рама 3)</t>
+          <t>Затяжка крайней рамы</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.434</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>5 (12 м)</t>
+          <t>4 (6 м)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>5.780 + 5.780</t>
+          <t>4.540</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (край → рама 3)</t>
+          <t>Нижний пояс боковой фермы</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.434</v>
+        <v>1.457</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>6 (12 м)</t>
+          <t>5 (6 м)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>5.780 + 5.780</t>
+          <t>4.540</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (край → рама 3)</t>
+          <t>Нижний пояс боковой фермы</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.434</v>
+        <v>1.457</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>7 (12 м)</t>
+          <t>6 (6 м)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>5.780 + 5.780</t>
+          <t>2.403 + 2.403</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (край → рама 3)</t>
+          <t>Раскос боковой фермы</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.434</v>
+        <v>1.188</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>8 (12 м)</t>
+          <t>7 (6 м)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>5.780 + 5.780</t>
+          <t>2.403 + 2.403</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (край → рама 3)</t>
+          <t>Раскос боковой фермы</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.434</v>
+        <v>1.188</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>9 (12 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>5.780 + 5.780</t>
+          <t>0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.950</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (край → рама 3)</t>
+          <t>Подкос фермы</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.434</v>
+        <v>0.282</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10 (12 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>5.780 + 5.780</t>
+          <t>0.598 + 0.598 + 0.598</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (край → рама 3)</t>
+          <t>Подвеска у конька</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0.434</v>
+        <v>4.197</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□30×30×2</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>11 (12 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>5.780 + 5.780</t>
+          <t>0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (край → рама 3)</t>
+          <t>Вкладыш стыка обрешётины</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.434</v>
+        <v>3.734</v>
       </c>
     </row>
     <row r="22">
@@ -2187,21 +2239,21 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>12 (12 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1.200 + 1.200 + 1.200 + 1.200 + 1.200 + 1.200 + 1.200 + 1.200 + 1.200</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (рама 3 → край)</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1.173</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="23">
@@ -2212,21 +2264,21 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>13 (12 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.200 + 1.200 + 1.200 + 1.200 + 1.200 + 1.200 + 1.200 + 1.200 + 1.200</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (рама 3 → край)</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1.173</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="24">
@@ -2237,45 +2289,670 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>14 (6 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1.200 + 1.200 + 1.200 + 1.200</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (рама 3 → край)</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1.188</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>4 (6 м)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>5 (6 м)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>6 (6 м)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>7 (6 м)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>8 (6 м)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>9 (6 м)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>10 (6 м)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>11 (6 м)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>12 (6 м)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>13 (6 м)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>14 (6 м)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>15 (6 м)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>16 (6 м)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>17 (6 м)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>18 (6 м)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>19 (6 м)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>20 (6 м)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>21 (6 м)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>22 (6 м)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>5.490</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>0.507</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>23 (6 м)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>0.028</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>24 (6 м)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>0.028</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>25 (6 м)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>0.028</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>26 (6 м)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>0.028</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>27 (6 м)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>0.028</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>28 (6 м)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1.490 + 1.490</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>3.014</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>□60×60×3</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>1 (6 м)</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>0.113 + 0.113</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>Стойка-вставка</t>
         </is>
       </c>
-      <c r="E25" t="n">
+      <c r="E50" t="n">
         <v>5.768</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Bar lengths from the full price list (column L): 100x60 12 m only, 60x60x3 6/12 m, others 6 m; cutting plan and texts updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X6AG5Fdm1RBCCrsAG1aTU6
</commit_message>
<xml_diff>
--- a/output/smeta_optimized.xlsx
+++ b/output/smeta_optimized.xlsx
@@ -1694,7 +1694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1739,21 +1739,21 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>1 (12 м)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>4.013</t>
+          <t>4.013 + 3.993 + 3.833</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Колонна П3</t>
+          <t>Колонна Л3; Колонна П1; Колонна П3</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1.984</v>
+        <v>0.152</v>
       </c>
     </row>
     <row r="3">
@@ -1764,77 +1764,77 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>2 (12 м)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>3.993</t>
+          <t>3.803</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Колонна Л3</t>
+          <t>Колонна Л1</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2.004</v>
+        <v>8.194000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>□100×60×4</t>
+          <t>□100×60×3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3 (6 м)</t>
+          <t>1 (12 м)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.833</t>
+          <t>3.710 + 3.710 + 3.710</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Колонна П1</t>
+          <t>Стропило длинное (свес 0.90)</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>2.164</v>
+        <v>0.861</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>□100×60×4</t>
+          <t>□100×60×3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4 (6 м)</t>
+          <t>2 (12 м)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.803</t>
+          <t>3.199 + 3.199 + 3.199</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Колонна Л1</t>
+          <t>Стропило короткое (свес 0.40)</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2.194</v>
+        <v>2.394</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>□100×60×3</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1844,22 +1844,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.710</t>
+          <t>5.397</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Стропило длинное (свес 0.90)</t>
+          <t>Затяжка средней рамы</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2.287</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>□100×60×3</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1869,22 +1869,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>3.710</t>
+          <t>5.357</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Стропило длинное (свес 0.90)</t>
+          <t>Затяжка крайней рамы</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>2.287</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>□100×60×3</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1894,22 +1894,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3.710</t>
+          <t>5.357</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Стропило длинное (свес 0.90)</t>
+          <t>Затяжка крайней рамы</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>2.287</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>□100×60×3</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1919,22 +1919,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>3.199</t>
+          <t>4.540</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Стропило короткое (свес 0.40)</t>
+          <t>Нижний пояс боковой фермы</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>2.798</v>
+        <v>1.457</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>□100×60×3</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1944,22 +1944,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>3.199</t>
+          <t>4.540</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Стропило короткое (свес 0.40)</t>
+          <t>Нижний пояс боковой фермы</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2.798</v>
+        <v>1.457</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>□100×60×3</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1969,16 +1969,16 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3.199</t>
+          <t>2.403 + 2.403</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Стропило короткое (свес 0.40)</t>
+          <t>Раскос боковой фермы</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2.798</v>
+        <v>1.188</v>
       </c>
     </row>
     <row r="12">
@@ -1989,246 +1989,246 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>7 (6 м)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>5.397</t>
+          <t>2.403 + 2.403</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Затяжка средней рамы</t>
+          <t>Раскос боковой фермы</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.6</v>
+        <v>1.188</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>5.357</t>
+          <t>0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.950</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Затяжка крайней рамы</t>
+          <t>Подкос фермы</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.64</v>
+        <v>0.282</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>3 (6 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5.357</t>
+          <t>0.598 + 0.598 + 0.598</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Затяжка крайней рамы</t>
+          <t>Подвеска у конька</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.64</v>
+        <v>4.197</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□30×30×2</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>4 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.540</t>
+          <t>0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы</t>
+          <t>Вкладыш стыка обрешётины</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>1.457</v>
+        <v>3.734</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>5 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>4.540</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1.457</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>6 (6 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2.403 + 2.403</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>1.188</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7 (6 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2.403 + 2.403</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1.188</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>□20×20×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>4 (6 м)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.950</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Подкос фермы</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.282</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>□20×20×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>5 (6 м)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.598 + 0.598 + 0.598</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Подвеска у конька</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4.197</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>□30×30×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>6 (6 м)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Вкладыш стыка обрешётины</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>3.734</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="22">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>7 (6 м)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>8 (6 м)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>3 (6 м)</t>
+          <t>9 (6 м)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>4 (6 м)</t>
+          <t>10 (6 м)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>5 (6 м)</t>
+          <t>11 (6 м)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>6 (6 м)</t>
+          <t>12 (6 м)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>7 (6 м)</t>
+          <t>13 (6 м)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>8 (6 м)</t>
+          <t>14 (6 м)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>9 (6 м)</t>
+          <t>15 (6 м)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10 (6 м)</t>
+          <t>16 (6 м)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>11 (6 м)</t>
+          <t>17 (6 м)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>12 (6 м)</t>
+          <t>18 (6 м)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2539,7 +2539,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>13 (6 м)</t>
+          <t>19 (6 м)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>14 (6 м)</t>
+          <t>20 (6 м)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2589,7 +2589,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>15 (6 м)</t>
+          <t>21 (6 м)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>16 (6 м)</t>
+          <t>22 (6 м)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2639,21 +2639,21 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>17 (6 м)</t>
+          <t>23 (6 м)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.507</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="39">
@@ -2664,21 +2664,21 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>18 (6 м)</t>
+          <t>24 (6 м)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0.507</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="40">
@@ -2689,21 +2689,21 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>19 (6 м)</t>
+          <t>25 (6 м)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.507</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="41">
@@ -2714,21 +2714,21 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>20 (6 м)</t>
+          <t>26 (6 м)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0.507</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="42">
@@ -2739,21 +2739,21 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>21 (6 м)</t>
+          <t>27 (6 м)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.507</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="43">
@@ -2764,195 +2764,45 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>22 (6 м)</t>
+          <t>28 (6 м)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.490 + 1.490</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>0.507</v>
+        <v>3.014</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□60×60×3</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>23 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+          <t>0.113 + 0.113</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Стойка-вставка</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.028</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>□35×35×2</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>24 (6 м)</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
-        </is>
-      </c>
-      <c r="E45" t="n">
-        <v>0.028</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>□35×35×2</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>25 (6 м)</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
-        </is>
-      </c>
-      <c r="E46" t="n">
-        <v>0.028</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>□35×35×2</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>26 (6 м)</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
-        </is>
-      </c>
-      <c r="E47" t="n">
-        <v>0.028</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>□35×35×2</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>27 (6 м)</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
-        </is>
-      </c>
-      <c r="E48" t="n">
-        <v>0.028</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>□35×35×2</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>28 (6 м)</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>1.490 + 1.490</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
-        </is>
-      </c>
-      <c r="E49" t="n">
-        <v>3.014</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>□60×60×3</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>1 (6 м)</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>0.113 + 0.113</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Стойка-вставка</t>
-        </is>
-      </c>
-      <c r="E50" t="n">
         <v>5.768</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adopt gable edge beam 60x60x2 with 30x30x2 knee braces (installer load, DBN 6.10): model, node G drawing and plan, fab details, cutting plan, report, reply and PDFs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X6AG5Fdm1RBCCrsAG1aTU6
</commit_message>
<xml_diff>
--- a/output/smeta_optimized.xlsx
+++ b/output/smeta_optimized.xlsx
@@ -480,7 +480,7 @@
         <v>75812</v>
       </c>
       <c r="C2" t="n">
-        <v>45534</v>
+        <v>49265</v>
       </c>
       <c r="D2">
         <f>C2-B2</f>
@@ -678,7 +678,7 @@
         <v>5500</v>
       </c>
       <c r="C11" t="n">
-        <v>3911</v>
+        <v>4279</v>
       </c>
       <c r="D11">
         <f>C11-B11</f>
@@ -700,7 +700,7 @@
         <v>6600</v>
       </c>
       <c r="C12" t="n">
-        <v>4377</v>
+        <v>5481</v>
       </c>
       <c r="D12">
         <f>C12-B12</f>
@@ -810,7 +810,7 @@
         <v>24000</v>
       </c>
       <c r="C17" t="n">
-        <v>17121</v>
+        <v>21216</v>
       </c>
       <c r="D17">
         <f>C17-B17</f>
@@ -832,7 +832,7 @@
         <v>7000</v>
       </c>
       <c r="C18" t="n">
-        <v>4977</v>
+        <v>5446</v>
       </c>
       <c r="D18">
         <f>C18-B18</f>
@@ -854,7 +854,7 @@
         <v>15000</v>
       </c>
       <c r="C19" t="n">
-        <v>10700</v>
+        <v>13260</v>
       </c>
       <c r="D19">
         <f>C19-B19</f>
@@ -920,7 +920,7 @@
         <v>7000</v>
       </c>
       <c r="C22" t="n">
-        <v>4993</v>
+        <v>6188</v>
       </c>
       <c r="D22">
         <f>C22-B22</f>
@@ -961,7 +961,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Масса металла: было 1226 кг, стало 763 кг; площадь окраски 57.6 → 40.9 м²; швы 37.6 → 24.9 м; деталей 84 → 74.</t>
+          <t>Масса металла: было 1226 кг, стало 822 кг; площадь окраски 57.6 → 44.8 м²; швы 37.6 → 31.2 м; деталей 84 → 82.</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1055,159 +1055,186 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>□100×60×3</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Стропила</t>
+          <t>Затяжки, Нижний пояс боковой фермы, Раскосы боковой фермы, Торцевая обвязка обрешётки</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.75</v>
+        <v>49.19</v>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E3" t="n">
-        <v>146.7</v>
+        <v>175.2</v>
       </c>
       <c r="F3" t="n">
-        <v>428</v>
+        <v>226</v>
       </c>
       <c r="G3" t="n">
-        <v>8879</v>
+        <v>11117</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>□100×60×4</t>
+          <t>□100×60×3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Колонны</t>
+          <t>Стропила</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>15.65</v>
+        <v>20.75</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E4" t="n">
-        <v>144.4</v>
+        <v>146.7</v>
       </c>
       <c r="F4" t="n">
-        <v>540</v>
+        <v>428</v>
       </c>
       <c r="G4" t="n">
-        <v>8453</v>
+        <v>8879</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□100×60×4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Затяжки, Нижний пояс боковой фермы, Раскосы боковой фермы</t>
+          <t>Колонны</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>35.41</v>
+        <v>15.65</v>
       </c>
       <c r="D5" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>126.1</v>
+        <v>144.4</v>
       </c>
       <c r="F5" t="n">
-        <v>226</v>
+        <v>540</v>
       </c>
       <c r="G5" t="n">
-        <v>8003</v>
+        <v>8453</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>□20×20×2</t>
+          <t>□30×30×2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Подвеска (стойка у конька), Подкосы фермы</t>
+          <t>Подкосы торцевой обвязки</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>8.69</v>
+        <v>5.71</v>
       </c>
       <c r="D6" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>9.1</v>
+        <v>9.6</v>
       </c>
       <c r="F6" t="n">
-        <v>67.40000000000001</v>
+        <v>108</v>
       </c>
       <c r="G6" t="n">
-        <v>586</v>
+        <v>617</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>□60×60×3</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Стойка-вставка средней рамы</t>
+          <t>Подвеска (стойка у конька), Подкосы фермы</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.3</v>
+        <v>8.69</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>1.5</v>
+        <v>9.1</v>
       </c>
       <c r="F7" t="n">
-        <v>315</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>94</v>
+        <v>586</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ИТОГО трубы</t>
-        </is>
-      </c>
-      <c r="C8">
-        <f>SUM(C2:C7)</f>
-        <v/>
-      </c>
-      <c r="E8">
-        <f>SUM(E2:E7)</f>
-        <v/>
-      </c>
-      <c r="G8">
-        <f>SUM(G2:G7)</f>
-        <v/>
+          <t>□60×60×3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Стойка-вставка средней рамы</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>315</v>
+      </c>
+      <c r="G8" t="n">
+        <v>94</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>ИТОГО трубы</t>
+        </is>
+      </c>
+      <c r="C9">
+        <f>SUM(C2:C8)</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>SUM(E2:E8)</f>
+        <v/>
+      </c>
+      <c r="G9">
+        <f>SUM(G2:G8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Пластины (фасонки, крышки колонн): 30.1 кг × 55 грн/кг</t>
         </is>
@@ -1224,7 +1251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1608,7 +1635,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы</t>
+          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1617,24 +1644,24 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2.403</v>
+        <v>3.698</v>
       </c>
       <c r="D15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E15" t="n">
-        <v>34.2</v>
+        <v>26.3</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>оба торца — горизонтальные резы под 20.7° к оси (рез по грани 170 мм): низ — на пояс, верх — под столик</t>
+          <t>у карниза — прямой рез, у конька — вертикальный рез (78° к оси) встык со второй половиной</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы</t>
+          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1643,41 +1670,145 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4.54</v>
+        <v>3.186</v>
       </c>
       <c r="D16" t="n">
         <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>32.3</v>
+        <v>22.7</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>оба торца — прямые; по фактическому расстоянию между гранями колонн</t>
+          <t>у карниза — прямой рез, у конька — вертикальный рез (78° к оси) встык со второй половиной</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Стойка-вставка</t>
+          <t>Подкос торцевой обвязки, задний свес</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>□60×60×3</t>
+          <t>□30×30×2</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.113</v>
+        <v>1.362</v>
       </c>
       <c r="D17" t="n">
         <v>2</v>
       </c>
       <c r="E17" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>низ — вертикальный рез к грани колонны на +2.10, верх — горизонтальный рез под обвязку (45° к горизонту)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Подкос торцевой обвязки, передний свес</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>□30×30×2</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1.348</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>низ — вертикальный рез к грани колонны на +2.10, верх — горизонтальный рез под обвязку (45° к горизонту)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Раскос боковой фермы</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>□60×60×2</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2.403</v>
+      </c>
+      <c r="D19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E19" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>оба торца — горизонтальные резы под 20.7° к оси (рез по грани 170 мм): низ — на пояс, верх — под столик</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Нижний пояс боковой фермы</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>□60×60×2</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>оба торца — прямые; по фактическому расстоянию между гранями колонн</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Стойка-вставка</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>□60×60×3</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="n">
         <v>1.2</v>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>низ — прямой (встаёт на столик фермы), верх — под 12°</t>
         </is>
@@ -1694,7 +1825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1969,16 +2100,16 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2.403 + 2.403</t>
+          <t>3.698</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы</t>
+          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1.188</v>
+        <v>2.299</v>
       </c>
     </row>
     <row r="12">
@@ -1994,97 +2125,97 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.403 + 2.403</t>
+          <t>3.698</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы</t>
+          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1.188</v>
+        <v>2.299</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>□20×20×2</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>8 (6 м)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.950</t>
+          <t>3.186 + 2.403</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Подкос фермы</t>
+          <t>Раскос боковой фермы; Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.282</v>
+        <v>0.405</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>□20×20×2</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>9 (6 м)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0.598 + 0.598 + 0.598</t>
+          <t>3.186 + 2.403</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Подвеска у конька</t>
+          <t>Раскос боковой фермы; Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>4.197</v>
+        <v>0.405</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>□30×30×2</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>10 (6 м)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100</t>
+          <t>2.403 + 2.403</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Вкладыш стыка обрешётины</t>
+          <t>Раскос боковой фермы</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>3.734</v>
+        <v>1.188</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2094,22 +2225,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.950</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Подкос фермы</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.507</v>
+        <v>0.282</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2119,66 +2250,66 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>0.598 + 0.598 + 0.598</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Подвеска у конька</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.507</v>
+        <v>4.197</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□30×30×2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>3 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.362 + 1.362 + 1.348 + 1.348 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Вкладыш стыка обрешётины; Подкос торцевой обвязки, задний свес; Подкос торцевой обвязки, передний свес</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.507</v>
+        <v>0.053</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□30×30×2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>4 (6 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Вкладыш стыка обрешётины</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.507</v>
+        <v>4.249</v>
       </c>
     </row>
     <row r="20">
@@ -2189,7 +2320,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>5 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2214,7 +2345,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>6 (6 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2239,7 +2370,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>7 (6 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2264,7 +2395,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>8 (6 м)</t>
+          <t>4 (6 м)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2289,7 +2420,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>9 (6 м)</t>
+          <t>5 (6 м)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2314,7 +2445,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10 (6 м)</t>
+          <t>6 (6 м)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2339,7 +2470,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>11 (6 м)</t>
+          <t>7 (6 м)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2364,7 +2495,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>12 (6 м)</t>
+          <t>8 (6 м)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2389,7 +2520,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>13 (6 м)</t>
+          <t>9 (6 м)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2414,7 +2545,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>14 (6 м)</t>
+          <t>10 (6 м)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2439,7 +2570,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>15 (6 м)</t>
+          <t>11 (6 м)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2464,7 +2595,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>16 (6 м)</t>
+          <t>12 (6 м)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2489,7 +2620,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>17 (6 м)</t>
+          <t>13 (6 м)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2514,7 +2645,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>18 (6 м)</t>
+          <t>14 (6 м)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2539,7 +2670,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>19 (6 м)</t>
+          <t>15 (6 м)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2564,7 +2695,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>20 (6 м)</t>
+          <t>16 (6 м)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2589,7 +2720,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>21 (6 м)</t>
+          <t>17 (6 м)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2614,7 +2745,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>22 (6 м)</t>
+          <t>18 (6 м)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2639,21 +2770,21 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>23 (6 м)</t>
+          <t>19 (6 м)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.028</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="39">
@@ -2664,21 +2795,21 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>24 (6 м)</t>
+          <t>20 (6 м)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0.028</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="40">
@@ -2689,21 +2820,21 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>25 (6 м)</t>
+          <t>21 (6 м)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.028</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="41">
@@ -2714,21 +2845,21 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>26 (6 м)</t>
+          <t>22 (6 м)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0.028</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="42">
@@ -2739,7 +2870,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>27 (6 м)</t>
+          <t>23 (6 м)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2764,12 +2895,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>28 (6 м)</t>
+          <t>24 (6 м)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>1.490 + 1.490</t>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2778,31 +2909,131 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>3.014</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>25 (6 м)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>0.028</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>26 (6 м)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>0.028</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>27 (6 м)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>0.028</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>□35×35×2</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>28 (6 м)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1.490 + 1.490</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>3.014</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>□60×60×3</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>1 (6 м)</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>0.113 + 0.113</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>Стойка-вставка</t>
         </is>
       </c>
-      <c r="E44" t="n">
+      <c r="E48" t="n">
         <v>5.768</v>
       </c>
     </row>
@@ -3493,7 +3724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3554,16 +3785,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>24.1</v>
+        <v>24.33</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>2.511</v>
+        <v>2.423</v>
       </c>
       <c r="F2" t="n">
-        <v>0.857</v>
+        <v>0.855</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -3583,20 +3814,20 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.09</v>
+        <v>26.11</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8</v>
+        <v>0.98</v>
       </c>
       <c r="E3" t="n">
-        <v>4.073</v>
+        <v>3.715</v>
       </c>
       <c r="F3" t="n">
-        <v>0.959</v>
+        <v>0.902</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>устойчивость [D+S+0.9W+x]</t>
+          <t>устойчивость [D+S+0.9W+y]</t>
         </is>
       </c>
     </row>
@@ -3612,13 +3843,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.57</v>
+        <v>0.36</v>
       </c>
       <c r="D4" t="n">
-        <v>26.35</v>
+        <v>24.98</v>
       </c>
       <c r="E4" t="n">
-        <v>0.367</v>
+        <v>0.379</v>
       </c>
       <c r="F4" t="n">
         <v>0.772</v>
@@ -3644,17 +3875,17 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>1.68</v>
+        <v>1.54</v>
       </c>
       <c r="E5" t="n">
-        <v>0.021</v>
+        <v>0.011</v>
       </c>
       <c r="F5" t="n">
-        <v>0.31</v>
+        <v>0.284</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>узел kp→tie: продавливание грани пояса N=1.7 кН, NRd=5.4 кН</t>
+          <t>узел kp→tie: продавливание грани пояса N=1.5 кН, NRd=5.4 кН</t>
         </is>
       </c>
     </row>
@@ -3670,16 +3901,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5.61</v>
+        <v>5.53</v>
       </c>
       <c r="D6" t="n">
-        <v>2.78</v>
+        <v>2.85</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01</v>
+        <v>0.008</v>
       </c>
       <c r="F6" t="n">
-        <v>0.896</v>
+        <v>0.893</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -3699,27 +3930,27 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.88</v>
+        <v>1.46</v>
       </c>
       <c r="D7" t="n">
-        <v>2.1</v>
+        <v>3.85</v>
       </c>
       <c r="E7" t="n">
-        <v>0.438</v>
+        <v>0.274</v>
       </c>
       <c r="F7" t="n">
-        <v>0.887</v>
+        <v>0.633</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>прочность [D+S+0.9W+x]</t>
+          <t>устойчивость [D+S+0.9W+y]</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Раскосы боковой фермы</t>
+          <t>Торцевая обвязка обрешётки</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3728,76 +3959,134 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>20.87</v>
+        <v>1.44</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="E8" t="n">
-        <v>0.166</v>
+        <v>0.601</v>
       </c>
       <c r="F8" t="n">
         <v>0.643</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>стенка c/t [D+S]</t>
+          <t>стенка c/t изг. [D+S]</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы</t>
+          <t>Подкосы торцевой обвязки</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□30×30×2</t>
         </is>
       </c>
       <c r="C9" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="D9" t="n">
         <v>0</v>
       </c>
-      <c r="D9" t="n">
-        <v>17.85</v>
-      </c>
       <c r="E9" t="n">
-        <v>0.12</v>
+        <v>0.092</v>
       </c>
       <c r="F9" t="n">
-        <v>0.643</v>
+        <v>0.706</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>стенка c/t изг. [D+S]</t>
+          <t>гибкость [D+S+0.9W+x]</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Стойка-вставка средней рамы</t>
+          <t>Раскосы боковой фермы</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>□60×60×3</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>13.97</v>
+        <v>22.55</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>1.95</v>
+        <v>0.254</v>
       </c>
       <c r="F10" t="n">
-        <v>0.83</v>
+        <v>0.643</v>
       </c>
       <c r="G10" t="inlineStr">
+        <is>
+          <t>стенка c/t [D+S]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Нижний пояс боковой фермы</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>□60×60×2</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>18.67</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.136</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.643</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>стенка c/t изг. [D+S]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Стойка-вставка средней рамы</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>□60×60×3</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2.123</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.904</v>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>устойчивость [D+S]</t>
         </is>

</xml_diff>

<commit_message>
Edge beam 50×30×2 without knee braces on stiffer eave (50×30×2) and ridge (60×60×2) laths
- eave laths 50×30×2 on edge: 15 mm higher than ordinary laths, the raise metal tile needs at the eave
- edge beam effective length in the vertical plane from its own buckling on elastic lath supports
- node G redrawn (eave and ridge sections), fabrication details, cutting, report, xlsx, PDFs,
  contractor reply point 5, decisions log and README updated; total 197 751

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X6AG5Fdm1RBCCrsAG1aTU6
</commit_message>
<xml_diff>
--- a/output/smeta_optimized.xlsx
+++ b/output/smeta_optimized.xlsx
@@ -480,7 +480,7 @@
         <v>75812</v>
       </c>
       <c r="C2" t="n">
-        <v>49265</v>
+        <v>48614</v>
       </c>
       <c r="D2">
         <f>C2-B2</f>
@@ -678,7 +678,7 @@
         <v>5500</v>
       </c>
       <c r="C11" t="n">
-        <v>4279</v>
+        <v>4206</v>
       </c>
       <c r="D11">
         <f>C11-B11</f>
@@ -700,7 +700,7 @@
         <v>6600</v>
       </c>
       <c r="C12" t="n">
-        <v>5481</v>
+        <v>5235</v>
       </c>
       <c r="D12">
         <f>C12-B12</f>
@@ -810,7 +810,7 @@
         <v>24000</v>
       </c>
       <c r="C17" t="n">
-        <v>21216</v>
+        <v>20096</v>
       </c>
       <c r="D17">
         <f>C17-B17</f>
@@ -832,7 +832,7 @@
         <v>7000</v>
       </c>
       <c r="C18" t="n">
-        <v>5446</v>
+        <v>5353</v>
       </c>
       <c r="D18">
         <f>C18-B18</f>
@@ -854,7 +854,7 @@
         <v>15000</v>
       </c>
       <c r="C19" t="n">
-        <v>13260</v>
+        <v>12560</v>
       </c>
       <c r="D19">
         <f>C19-B19</f>
@@ -920,7 +920,7 @@
         <v>7000</v>
       </c>
       <c r="C22" t="n">
-        <v>6188</v>
+        <v>5861</v>
       </c>
       <c r="D22">
         <f>C22-B22</f>
@@ -961,7 +961,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Масса металла: было 1226 кг, стало 822 кг; площадь окраски 57.6 → 44.8 м²; швы 37.6 → 31.2 м; деталей 84 → 82.</t>
+          <t>Масса металла: было 1226 кг, стало 810 кг; площадь окраски 57.6 → 44.0 м²; швы 37.6 → 29.8 м; деталей 84 → 78.</t>
         </is>
       </c>
     </row>
@@ -1037,19 +1037,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>153.69</v>
+        <v>132.73</v>
       </c>
       <c r="D2" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="E2" t="n">
-        <v>306.1</v>
+        <v>264.3</v>
       </c>
       <c r="F2" t="n">
         <v>127</v>
       </c>
       <c r="G2" t="n">
-        <v>19519</v>
+        <v>16857</v>
       </c>
     </row>
     <row r="3">
@@ -1060,23 +1060,23 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Затяжки, Нижний пояс боковой фермы, Раскосы боковой фермы, Торцевая обвязка обрешётки</t>
+          <t>Затяжки, Коньковая обрешётина, Нижний пояс боковой фермы, Раскосы боковой фермы</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>49.19</v>
+        <v>42.4</v>
       </c>
       <c r="D3" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E3" t="n">
-        <v>175.2</v>
+        <v>151</v>
       </c>
       <c r="F3" t="n">
         <v>226</v>
       </c>
       <c r="G3" t="n">
-        <v>11117</v>
+        <v>9582</v>
       </c>
     </row>
     <row r="4">
@@ -1136,28 +1136,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>□30×30×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Подкосы торцевой обвязки</t>
+          <t>Карнизные обрешётины, Торцевая обвязка обрешётки</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5.71</v>
+        <v>27.75</v>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E6" t="n">
-        <v>9.6</v>
+        <v>64</v>
       </c>
       <c r="F6" t="n">
-        <v>108</v>
+        <v>150</v>
       </c>
       <c r="G6" t="n">
-        <v>617</v>
+        <v>4163</v>
       </c>
     </row>
     <row r="7">
@@ -1251,7 +1251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1569,14 +1569,14 @@
         <v>0.1</v>
       </c>
       <c r="D12" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E12" t="n">
-        <v>3.7</v>
+        <v>3.2</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>отрезок трубы внутрь стыка, по 50 мм в каждую часть</t>
+          <t>отрезок трубы внутрь стыка, по 50 мм в каждую часть (по желанию)</t>
         </is>
       </c>
     </row>
@@ -1595,10 +1595,10 @@
         <v>5.49</v>
       </c>
       <c r="D13" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E13" t="n">
-        <v>240.5</v>
+        <v>207.7</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         <v>1.49</v>
       </c>
       <c r="D14" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E14" t="n">
-        <v>65.3</v>
+        <v>56.4</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1650,7 +1650,7 @@
         <v>2</v>
       </c>
       <c r="E15" t="n">
-        <v>26.3</v>
+        <v>17.1</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1676,7 +1676,7 @@
         <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>22.7</v>
+        <v>14.7</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1687,59 +1687,59 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Подкос торцевой обвязки, задний свес</t>
+          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>□30×30×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.362</v>
+        <v>5.49</v>
       </c>
       <c r="D17" t="n">
         <v>2</v>
       </c>
       <c r="E17" t="n">
-        <v>4.6</v>
+        <v>25.3</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>низ — вертикальный рез к грани колонны на +2.10, верх — горизонтальный рез под обвязку (45° к горизонту)</t>
+          <t>торцы прямые; стык с частью 2 — в пролёте, в 290 мм от стропила рамы 3 (на вкладыше, см. узлы)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Подкос торцевой обвязки, передний свес</t>
+          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>□30×30×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1.348</v>
+        <v>1.49</v>
       </c>
       <c r="D18" t="n">
         <v>2</v>
       </c>
       <c r="E18" t="n">
-        <v>4.5</v>
+        <v>6.9</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>низ — вертикальный рез к грани колонны на +2.10, верх — горизонтальный рез под обвязку (45° к горизонту)</t>
+          <t>торцы прямые</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы</t>
+          <t>Коньковая обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1748,24 +1748,24 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2.403</v>
+        <v>5.49</v>
       </c>
       <c r="D19" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>34.2</v>
+        <v>19.6</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>оба торца — горизонтальные резы под 20.7° к оси (рез по грани 170 мм): низ — на пояс, верх — под столик</t>
+          <t>торцы прямые; стык с частью 2 — в пролёте, в 290 мм от стропила рамы 3 (на вкладыше, см. узлы)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы</t>
+          <t>Коньковая обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1774,41 +1774,93 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4.54</v>
+        <v>1.49</v>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>32.3</v>
+        <v>5.3</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>оба торца — прямые; по фактическому расстоянию между гранями колонн</t>
+          <t>торцы прямые</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>Раскос боковой фермы</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>□60×60×2</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2.403</v>
+      </c>
+      <c r="D21" t="n">
+        <v>4</v>
+      </c>
+      <c r="E21" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>оба торца — горизонтальные резы под 20.7° к оси (рез по грани 170 мм): низ — на пояс, верх — под столик</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Нижний пояс боковой фермы</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>□60×60×2</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>оба торца — прямые; по фактическому расстоянию между гранями колонн</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>Стойка-вставка</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>□60×60×3</t>
         </is>
       </c>
-      <c r="C21" t="n">
+      <c r="C23" t="n">
         <v>0.113</v>
       </c>
-      <c r="D21" t="n">
+      <c r="D23" t="n">
         <v>2</v>
       </c>
-      <c r="E21" t="n">
+      <c r="E23" t="n">
         <v>1.2</v>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>низ — прямой (встаёт на столик фермы), верх — под 12°</t>
         </is>
@@ -1975,16 +2027,16 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.397</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Затяжка средней рамы</t>
+          <t>Коньковая обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.6</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="7">
@@ -2000,16 +2052,16 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.357</t>
+          <t>5.397</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Затяжка крайней рамы</t>
+          <t>Затяжка средней рамы</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.64</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="8">
@@ -2050,16 +2102,16 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>4.540</t>
+          <t>5.357</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы</t>
+          <t>Затяжка крайней рамы</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>1.457</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="10">
@@ -2100,16 +2152,16 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3.698</t>
+          <t>4.540</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
+          <t>Нижний пояс боковой фермы</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2.299</v>
+        <v>1.457</v>
       </c>
     </row>
     <row r="12">
@@ -2125,16 +2177,16 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.698</t>
+          <t>2.403 + 2.403</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
+          <t>Раскос боковой фермы</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>2.299</v>
+        <v>1.188</v>
       </c>
     </row>
     <row r="13">
@@ -2150,16 +2202,16 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3.186 + 2.403</t>
+          <t>2.403 + 2.403</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы; Торцевая обвязка (по скату, под обрешёткой)</t>
+          <t>Раскос боковой фермы</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.405</v>
+        <v>1.188</v>
       </c>
     </row>
     <row r="14">
@@ -2175,41 +2227,41 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3.186 + 2.403</t>
+          <t>1.490</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы; Торцевая обвязка (по скату, под обрешёткой)</t>
+          <t>Коньковая обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.405</v>
+        <v>4.507</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.403 + 2.403</t>
+          <t>0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.950</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы</t>
+          <t>Подкос фермы</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>1.188</v>
+        <v>0.282</v>
       </c>
     </row>
     <row r="16">
@@ -2220,52 +2272,52 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.950</t>
+          <t>0.598 + 0.598 + 0.598</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Подкос фермы</t>
+          <t>Подвеска у конька</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.282</v>
+        <v>4.197</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>□20×20×2</t>
+          <t>□30×30×2</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.598 + 0.598 + 0.598</t>
+          <t>0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Подвеска у конька</t>
+          <t>Вкладыш стыка обрешётины</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>4.197</v>
+        <v>4.043</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>□30×30×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2275,22 +2327,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.362 + 1.362 + 1.348 + 1.348 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Вкладыш стыка обрешётины; Подкос торцевой обвязки, задний свес; Подкос торцевой обвязки, передний свес</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.053</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>□30×30×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2300,16 +2352,16 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Вкладыш стыка обрешётины</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>4.249</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="20">
@@ -2320,7 +2372,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2345,7 +2397,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>4 (6 м)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2370,7 +2422,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>3 (6 м)</t>
+          <t>5 (6 м)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2395,7 +2447,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>4 (6 м)</t>
+          <t>6 (6 м)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2420,7 +2472,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>5 (6 м)</t>
+          <t>7 (6 м)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2445,7 +2497,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>6 (6 м)</t>
+          <t>8 (6 м)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2470,7 +2522,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>7 (6 м)</t>
+          <t>9 (6 м)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2495,7 +2547,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>8 (6 м)</t>
+          <t>10 (6 м)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2520,7 +2572,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>9 (6 м)</t>
+          <t>11 (6 м)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2545,7 +2597,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10 (6 м)</t>
+          <t>12 (6 м)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2570,7 +2622,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>11 (6 м)</t>
+          <t>13 (6 м)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2595,7 +2647,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>12 (6 м)</t>
+          <t>14 (6 м)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2620,7 +2672,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>13 (6 м)</t>
+          <t>15 (6 м)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2645,7 +2697,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>14 (6 м)</t>
+          <t>16 (6 м)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2670,7 +2722,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>15 (6 м)</t>
+          <t>17 (6 м)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2695,7 +2747,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>16 (6 м)</t>
+          <t>18 (6 м)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2720,7 +2772,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>17 (6 м)</t>
+          <t>19 (6 м)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2745,21 +2797,21 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>18 (6 м)</t>
+          <t>20 (6 м)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.507</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="38">
@@ -2770,21 +2822,21 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>19 (6 м)</t>
+          <t>21 (6 м)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.507</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="39">
@@ -2795,21 +2847,21 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>20 (6 м)</t>
+          <t>22 (6 м)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0.507</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="40">
@@ -2820,21 +2872,21 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>21 (6 м)</t>
+          <t>23 (6 м)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.507</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="41">
@@ -2845,171 +2897,171 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>22 (6 м)</t>
+          <t>24 (6 м)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0.507</v>
+        <v>1.521</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>23 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.028</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>24 (6 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>0.028</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>25 (6 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+          <t>3.698 + 1.490</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край); Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.028</v>
+        <v>0.806</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>26 (6 м)</t>
+          <t>4 (6 м)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+          <t>3.698 + 1.490</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край); Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.028</v>
+        <v>0.806</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>27 (6 м)</t>
+          <t>5 (6 м)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+          <t>3.186</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.028</v>
+        <v>2.811</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>28 (6 м)</t>
+          <t>6 (6 м)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>1.490 + 1.490</t>
+          <t>3.186</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>3.014</v>
+        <v>2.811</v>
       </c>
     </row>
     <row r="48">
@@ -3445,7 +3497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3697,7 +3749,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -3710,6 +3762,72 @@
       <c r="G8" t="inlineStr">
         <is>
           <t>пластиковые заглушки 35×35</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Заглушка торца карнизной обрешётины и обвязки</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>50 × 30</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>торцы карнизных обрешётин (4) и обвязки у карниза (4)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>пластиковые заглушки 50×30</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Заглушка торца коньковой обрешётины</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>60 × 60</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>торцы коньковой обрешётины</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>пластиковые заглушки 60×60</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3785,16 +3903,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>24.33</v>
+        <v>24.29</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>2.423</v>
+        <v>2.481</v>
       </c>
       <c r="F2" t="n">
-        <v>0.855</v>
+        <v>0.853</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -3814,20 +3932,20 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>26.11</v>
+        <v>27.82</v>
       </c>
       <c r="D3" t="n">
-        <v>0.98</v>
+        <v>1.09</v>
       </c>
       <c r="E3" t="n">
-        <v>3.715</v>
+        <v>4.078</v>
       </c>
       <c r="F3" t="n">
-        <v>0.902</v>
+        <v>0.958</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>устойчивость [D+S+0.9W+y]</t>
+          <t>устойчивость [D+S+0.9W+x]</t>
         </is>
       </c>
     </row>
@@ -3843,13 +3961,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.36</v>
+        <v>0.31</v>
       </c>
       <c r="D4" t="n">
-        <v>24.98</v>
+        <v>26.26</v>
       </c>
       <c r="E4" t="n">
-        <v>0.379</v>
+        <v>0.37</v>
       </c>
       <c r="F4" t="n">
         <v>0.772</v>
@@ -3875,17 +3993,17 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>1.54</v>
+        <v>1.66</v>
       </c>
       <c r="E5" t="n">
-        <v>0.011</v>
+        <v>0.018</v>
       </c>
       <c r="F5" t="n">
-        <v>0.284</v>
+        <v>0.306</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>узел kp→tie: продавливание грани пояса N=1.5 кН, NRd=5.4 кН</t>
+          <t>узел kp→tie: продавливание грани пояса N=1.7 кН, NRd=5.4 кН</t>
         </is>
       </c>
     </row>
@@ -3901,16 +4019,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5.53</v>
+        <v>5.42</v>
       </c>
       <c r="D6" t="n">
-        <v>2.85</v>
+        <v>2.87</v>
       </c>
       <c r="E6" t="n">
-        <v>0.008</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>0.893</v>
+        <v>0.889</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -3930,20 +4048,20 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.46</v>
+        <v>1.75</v>
       </c>
       <c r="D7" t="n">
-        <v>3.85</v>
+        <v>0.85</v>
       </c>
       <c r="E7" t="n">
-        <v>0.274</v>
+        <v>0.453</v>
       </c>
       <c r="F7" t="n">
-        <v>0.633</v>
+        <v>0.949</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>устойчивость [D+S+0.9W+y]</t>
+          <t>устойчивость [D+S+0.9W-x]</t>
         </is>
       </c>
     </row>
@@ -3955,60 +4073,60 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1.44</v>
+        <v>1.3</v>
       </c>
       <c r="D8" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="E8" t="n">
-        <v>0.601</v>
+        <v>0.258</v>
       </c>
       <c r="F8" t="n">
-        <v>0.643</v>
+        <v>0.655</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>стенка c/t изг. [D+S]</t>
+          <t>устойчивость [D+S]</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Подкосы торцевой обвязки</t>
+          <t>Карнизные обрешётины</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>□30×30×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3.28</v>
+        <v>0.6</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="E9" t="n">
-        <v>0.092</v>
+        <v>0.51</v>
       </c>
       <c r="F9" t="n">
-        <v>0.706</v>
+        <v>0.734</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>гибкость [D+S+0.9W+x]</t>
+          <t>устойчивость [D+S+0.9W+x]</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Раскосы боковой фермы</t>
+          <t>Коньковая обрешётина</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4017,27 +4135,27 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>22.55</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>3.08</v>
       </c>
       <c r="E10" t="n">
-        <v>0.254</v>
+        <v>0.912</v>
       </c>
       <c r="F10" t="n">
         <v>0.643</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>стенка c/t [D+S]</t>
+          <t>стенка c/t изг. [D+S]</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы</t>
+          <t>Раскосы боковой фермы</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4046,47 +4164,76 @@
         </is>
       </c>
       <c r="C11" t="n">
+        <v>21.02</v>
+      </c>
+      <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="D11" t="n">
-        <v>18.67</v>
-      </c>
       <c r="E11" t="n">
-        <v>0.136</v>
+        <v>0.181</v>
       </c>
       <c r="F11" t="n">
         <v>0.643</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>стенка c/t изг. [D+S]</t>
+          <t>стенка c/t [D+S]</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Нижний пояс боковой фермы</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>□60×60×2</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>18.01</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.643</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>стенка c/t изг. [D+S]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Стойка-вставка средней рамы</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>□60×60×3</t>
         </is>
       </c>
-      <c r="C12" t="n">
-        <v>15.12</v>
-      </c>
-      <c r="D12" t="n">
+      <c r="C13" t="n">
+        <v>14</v>
+      </c>
+      <c r="D13" t="n">
         <v>0</v>
       </c>
-      <c r="E12" t="n">
-        <v>2.123</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0.904</v>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="E13" t="n">
+        <v>1.991</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.847</v>
+      </c>
+      <c r="G13" t="inlineStr">
         <is>
           <t>устойчивость [D+S]</t>
         </is>

</xml_diff>

<commit_message>
Customer offcuts 60×60×3: two truss diagonals, ridge lath short part and stubs cut from them
Offcut details are flagged in the parts list, packed into the offcuts in the cutting plan and
excluded from purchase and metal cost (total 196 233). Reply to contractor, decisions log and README updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X6AG5Fdm1RBCCrsAG1aTU6
</commit_message>
<xml_diff>
--- a/output/smeta_optimized.xlsx
+++ b/output/smeta_optimized.xlsx
@@ -480,7 +480,7 @@
         <v>75812</v>
       </c>
       <c r="C2" t="n">
-        <v>48614</v>
+        <v>47095</v>
       </c>
       <c r="D2">
         <f>C2-B2</f>
@@ -976,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1055,82 +1055,82 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□100×60×3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Затяжки, Коньковая обрешётина, Нижний пояс боковой фермы, Раскосы боковой фермы</t>
+          <t>Стропила</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>42.4</v>
+        <v>20.75</v>
       </c>
       <c r="D3" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E3" t="n">
-        <v>151</v>
+        <v>146.7</v>
       </c>
       <c r="F3" t="n">
-        <v>226</v>
+        <v>428</v>
       </c>
       <c r="G3" t="n">
-        <v>9582</v>
+        <v>8879</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>□100×60×3</t>
+          <t>□100×60×4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Стропила</t>
+          <t>Колонны</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>20.75</v>
+        <v>15.65</v>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>146.7</v>
+        <v>144.4</v>
       </c>
       <c r="F4" t="n">
-        <v>428</v>
+        <v>540</v>
       </c>
       <c r="G4" t="n">
-        <v>8879</v>
+        <v>8453</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>□100×60×4</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Колонны</t>
+          <t>Затяжки, Коньковая обрешётина, Нижний пояс боковой фермы, Раскосы боковой фермы</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>15.65</v>
+        <v>36.09</v>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E5" t="n">
-        <v>144.4</v>
+        <v>128.5</v>
       </c>
       <c r="F5" t="n">
-        <v>540</v>
+        <v>226</v>
       </c>
       <c r="G5" t="n">
-        <v>8453</v>
+        <v>8157</v>
       </c>
     </row>
     <row r="6">
@@ -1190,51 +1190,24 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>□60×60×3</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Стойка-вставка средней рамы</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E8" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F8" t="n">
-        <v>315</v>
-      </c>
-      <c r="G8" t="n">
-        <v>94</v>
+          <t>ИТОГО трубы</t>
+        </is>
+      </c>
+      <c r="C8">
+        <f>SUM(C2:C7)</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>SUM(E2:E7)</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>SUM(G2:G7)</f>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
-        <is>
-          <t>ИТОГО трубы</t>
-        </is>
-      </c>
-      <c r="C9">
-        <f>SUM(C2:C8)</f>
-        <v/>
-      </c>
-      <c r="E9">
-        <f>SUM(E2:E8)</f>
-        <v/>
-      </c>
-      <c r="G9">
-        <f>SUM(G2:G8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
         <is>
           <t>Пластины (фасонки, крышки колонн): 30.1 кг × 55 грн/кг</t>
         </is>
@@ -1251,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1765,12 +1738,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Коньковая обрешётина, часть 2 (стык → задний край)</t>
+          <t>Коньковая обрешётина, часть 2 (стык → задний край) — из обрезка заказчика</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□60×60×3</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1780,11 +1753,11 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>5.3</v>
+        <v>7.7</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>торцы прямые</t>
+          <t>торцы прямые; □60×60×3 вместо □60×60×2 — размеры и резы те же</t>
         </is>
       </c>
     </row>
@@ -1803,10 +1776,10 @@
         <v>2.403</v>
       </c>
       <c r="D21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E21" t="n">
-        <v>34.2</v>
+        <v>17.1</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1817,50 +1790,76 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы</t>
+          <t>Раскос боковой фермы — из обрезка заказчика</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□60×60×3</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4.54</v>
+        <v>2.403</v>
       </c>
       <c r="D22" t="n">
         <v>2</v>
       </c>
       <c r="E22" t="n">
-        <v>32.3</v>
+        <v>24.9</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>оба торца — прямые; по фактическому расстоянию между гранями колонн</t>
+          <t>оба торца — горизонтальные резы под 20.7° к оси (рез по грани 170 мм): низ — на пояс, верх — под столик; □60×60×3 вместо □60×60×2 — размеры и резы те же</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Стойка-вставка</t>
+          <t>Нижний пояс боковой фермы</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>□60×60×3</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.113</v>
+        <v>4.54</v>
       </c>
       <c r="D23" t="n">
         <v>2</v>
       </c>
       <c r="E23" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>оба торца — прямые; по фактическому расстоянию между гранями колонн</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Стойка-вставка — из обрезка заказчика</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>□60×60×3</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="D24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" t="n">
         <v>1.2</v>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>низ — прямой (встаёт на столик фермы), верх — под 12°</t>
         </is>
@@ -1877,7 +1876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1917,201 +1916,193 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>□100×60×4</t>
+          <t>□60×60×3 (обрезки заказчика)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1 (12 м)</t>
+          <t>обрезок 1.74 м</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>4.013 + 3.993 + 3.833</t>
+          <t>1.490 + 0.113 + 0.113</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Колонна Л3; Колонна П1; Колонна П3</t>
+          <t>Коньковая обрешётина, часть 2 (стык → задний край) — из обрезка заказчика; Стойка-вставка — из обрезка заказчика</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.152</v>
+        <v>0.015</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>□100×60×4</t>
+          <t>□60×60×3 (обрезки заказчика)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2 (12 м)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>3.803</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Колонна Л1</t>
-        </is>
-      </c>
+          <t>обрезок 2.05 м</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>8.194000000000001</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>□100×60×3</t>
+          <t>□60×60×3 (обрезки заказчика)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1 (12 м)</t>
+          <t>обрезок 2.70 м</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.710 + 3.710 + 3.710</t>
+          <t>2.403</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Стропило длинное (свес 0.90)</t>
+          <t>Раскос боковой фермы — из обрезка заказчика</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.861</v>
+        <v>0.294</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>□100×60×3</t>
+          <t>□60×60×3 (обрезки заказчика)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2 (12 м)</t>
+          <t>обрезок 2.80 м</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3.199 + 3.199 + 3.199</t>
+          <t>2.403</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Стропило короткое (свес 0.40)</t>
+          <t>Раскос боковой фермы — из обрезка заказчика</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2.394</v>
+        <v>0.394</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□100×60×4</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>1 (12 м)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>4.013 + 3.993 + 3.833</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Коньковая обрешётина, часть 1 (передний край → стык)</t>
+          <t>Колонна Л3; Колонна П1; Колонна П3</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.507</v>
+        <v>0.152</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□100×60×4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>2 (12 м)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5.397</t>
+          <t>3.803</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Затяжка средней рамы</t>
+          <t>Колонна Л1</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.6</v>
+        <v>8.194000000000001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□100×60×3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>3 (6 м)</t>
+          <t>1 (12 м)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>5.357</t>
+          <t>3.710 + 3.710 + 3.710</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Затяжка крайней рамы</t>
+          <t>Стропило длинное (свес 0.90)</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.64</v>
+        <v>0.861</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□100×60×3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>4 (6 м)</t>
+          <t>2 (12 м)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>5.357</t>
+          <t>3.199 + 3.199 + 3.199</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Затяжка крайней рамы</t>
+          <t>Стропило короткое (свес 0.40)</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.64</v>
+        <v>2.394</v>
       </c>
     </row>
     <row r="10">
@@ -2122,21 +2113,21 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>5 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>4.540</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы</t>
+          <t>Коньковая обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1.457</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="11">
@@ -2147,21 +2138,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>6 (6 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>4.540</t>
+          <t>5.397</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы</t>
+          <t>Затяжка средней рамы</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1.457</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="12">
@@ -2172,21 +2163,21 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>7 (6 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.403 + 2.403</t>
+          <t>5.357</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы</t>
+          <t>Затяжка крайней рамы</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1.188</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="13">
@@ -2197,21 +2188,21 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>8 (6 м)</t>
+          <t>4 (6 м)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.403 + 2.403</t>
+          <t>5.357</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы</t>
+          <t>Затяжка крайней рамы</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1.188</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="14">
@@ -2222,77 +2213,77 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9 (6 м)</t>
+          <t>5 (6 м)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.490</t>
+          <t>4.540</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Коньковая обрешётина, часть 2 (стык → задний край)</t>
+          <t>Нижний пояс боковой фермы</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>4.507</v>
+        <v>1.457</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>□20×20×2</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>6 (6 м)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.950</t>
+          <t>4.540</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Подкос фермы</t>
+          <t>Нижний пояс боковой фермы</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.282</v>
+        <v>1.457</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>□20×20×2</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>7 (6 м)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.598 + 0.598 + 0.598</t>
+          <t>2.403 + 2.403</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Подвеска у конька</t>
+          <t>Раскос боковой фермы</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>4.197</v>
+        <v>1.188</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>□30×30×2</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2302,66 +2293,66 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100</t>
+          <t>0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.950</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Вкладыш стыка обрешётины</t>
+          <t>Подкос фермы</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>4.043</v>
+        <v>0.282</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>0.598 + 0.598 + 0.598</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Подвеска у конька</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.507</v>
+        <v>4.197</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□30×30×2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Вкладыш стыка обрешётины</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.507</v>
+        <v>4.043</v>
       </c>
     </row>
     <row r="20">
@@ -2372,7 +2363,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>3 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2397,7 +2388,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>4 (6 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2422,7 +2413,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>5 (6 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2447,7 +2438,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>6 (6 м)</t>
+          <t>4 (6 м)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2472,7 +2463,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>7 (6 м)</t>
+          <t>5 (6 м)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2497,7 +2488,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>8 (6 м)</t>
+          <t>6 (6 м)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2522,7 +2513,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>9 (6 м)</t>
+          <t>7 (6 м)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2547,7 +2538,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>10 (6 м)</t>
+          <t>8 (6 м)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2572,7 +2563,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>11 (6 м)</t>
+          <t>9 (6 м)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2597,7 +2588,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>12 (6 м)</t>
+          <t>10 (6 м)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2622,7 +2613,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>13 (6 м)</t>
+          <t>11 (6 м)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2647,7 +2638,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>14 (6 м)</t>
+          <t>12 (6 м)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2672,7 +2663,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>15 (6 м)</t>
+          <t>13 (6 м)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2697,7 +2688,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>16 (6 м)</t>
+          <t>14 (6 м)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2722,7 +2713,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>17 (6 м)</t>
+          <t>15 (6 м)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2747,7 +2738,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>18 (6 м)</t>
+          <t>16 (6 м)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2772,7 +2763,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>19 (6 м)</t>
+          <t>17 (6 м)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2797,21 +2788,21 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>20 (6 м)</t>
+          <t>18 (6 м)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.028</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="38">
@@ -2822,21 +2813,21 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>21 (6 м)</t>
+          <t>19 (6 м)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.028</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="39">
@@ -2847,7 +2838,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>22 (6 м)</t>
+          <t>20 (6 м)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2872,7 +2863,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>23 (6 м)</t>
+          <t>21 (6 м)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2897,12 +2888,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>24 (6 м)</t>
+          <t>22 (6 м)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490</t>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2911,57 +2902,57 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>1.521</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>□50×30×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>23 (6 м)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.507</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>□50×30×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>24 (6 м)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>0.507</v>
+        <v>1.521</v>
       </c>
     </row>
     <row r="44">
@@ -2972,21 +2963,21 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>3 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>3.698 + 1.490</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край); Торцевая обвязка (по скату, под обрешёткой)</t>
+          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.806</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="45">
@@ -2997,21 +2988,21 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>4 (6 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>3.698 + 1.490</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край); Торцевая обвязка (по скату, под обрешёткой)</t>
+          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.806</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="46">
@@ -3022,21 +3013,21 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>5 (6 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>3.186</t>
+          <t>3.698 + 1.490</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
+          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край); Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>2.811</v>
+        <v>0.806</v>
       </c>
     </row>
     <row r="47">
@@ -3047,46 +3038,71 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>6 (6 м)</t>
+          <t>4 (6 м)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>3.186</t>
+          <t>3.698 + 1.490</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
+          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край); Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>2.811</v>
+        <v>0.806</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>□60×60×3</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>5 (6 м)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.113 + 0.113</t>
+          <t>3.186</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Стойка-вставка</t>
+          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>5.768</v>
+        <v>2.811</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>□50×30×2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>6 (6 м)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>3.186</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>2.811</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ridge hanger 30×30×2 (one 20×20 bar less); unused customer offcut not shown in documents
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X6AG5Fdm1RBCCrsAG1aTU6
</commit_message>
<xml_diff>
--- a/output/smeta_optimized.xlsx
+++ b/output/smeta_optimized.xlsx
@@ -480,7 +480,7 @@
         <v>75812</v>
       </c>
       <c r="C2" t="n">
-        <v>47095</v>
+        <v>47178</v>
       </c>
       <c r="D2">
         <f>C2-B2</f>
@@ -678,7 +678,7 @@
         <v>5500</v>
       </c>
       <c r="C11" t="n">
-        <v>4206</v>
+        <v>4213</v>
       </c>
       <c r="D11">
         <f>C11-B11</f>
@@ -700,7 +700,7 @@
         <v>6600</v>
       </c>
       <c r="C12" t="n">
-        <v>5235</v>
+        <v>5277</v>
       </c>
       <c r="D12">
         <f>C12-B12</f>
@@ -810,7 +810,7 @@
         <v>24000</v>
       </c>
       <c r="C17" t="n">
-        <v>20096</v>
+        <v>20153</v>
       </c>
       <c r="D17">
         <f>C17-B17</f>
@@ -832,7 +832,7 @@
         <v>7000</v>
       </c>
       <c r="C18" t="n">
-        <v>5353</v>
+        <v>5362</v>
       </c>
       <c r="D18">
         <f>C18-B18</f>
@@ -854,7 +854,7 @@
         <v>15000</v>
       </c>
       <c r="C19" t="n">
-        <v>12560</v>
+        <v>12596</v>
       </c>
       <c r="D19">
         <f>C19-B19</f>
@@ -920,7 +920,7 @@
         <v>7000</v>
       </c>
       <c r="C22" t="n">
-        <v>5861</v>
+        <v>5878</v>
       </c>
       <c r="D22">
         <f>C22-B22</f>
@@ -961,7 +961,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Масса металла: было 1226 кг, стало 810 кг; площадь окраски 57.6 → 44.0 м²; швы 37.6 → 29.8 м; деталей 84 → 78.</t>
+          <t>Масса металла: было 1226 кг, стало 812 кг; площадь окраски 57.6 → 44.1 м²; швы 37.6 → 30.0 м; деталей 84 → 78.</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1168,46 +1168,73 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Подвеска (стойка у конька), Подкосы фермы</t>
+          <t>Подкосы фермы</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>8.69</v>
+        <v>6.65</v>
       </c>
       <c r="D7" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E7" t="n">
-        <v>9.1</v>
+        <v>7</v>
       </c>
       <c r="F7" t="n">
         <v>67.40000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>586</v>
+        <v>448</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ИТОГО трубы</t>
-        </is>
-      </c>
-      <c r="C8">
-        <f>SUM(C2:C7)</f>
-        <v/>
-      </c>
-      <c r="E8">
-        <f>SUM(E2:E7)</f>
-        <v/>
-      </c>
-      <c r="G8">
-        <f>SUM(G2:G7)</f>
-        <v/>
+          <t>□30×30×2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Подвеска (стойка у конька)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F8" t="n">
+        <v>108</v>
+      </c>
+      <c r="G8" t="n">
+        <v>221</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>ИТОГО трубы</t>
+        </is>
+      </c>
+      <c r="C9">
+        <f>SUM(C2:C8)</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>SUM(E2:E8)</f>
+        <v/>
+      </c>
+      <c r="G9">
+        <f>SUM(G2:G8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Пластины (фасонки, крышки колонн): 30.1 кг × 55 грн/кг</t>
         </is>
@@ -1483,7 +1510,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>□20×20×2</t>
+          <t>□30×30×2</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1493,7 +1520,7 @@
         <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>1.9</v>
+        <v>3</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1876,7 +1903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1946,13 +1973,21 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>обрезок 2.05 м</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
+          <t>обрезок 2.70 м</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2.403</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Раскос боковой фермы — из обрезка заказчика</t>
+        </is>
+      </c>
       <c r="E3" t="n">
-        <v>2.05</v>
+        <v>0.294</v>
       </c>
     </row>
     <row r="4">
@@ -1963,7 +1998,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>обрезок 2.70 м</t>
+          <t>обрезок 2.80 м</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1977,32 +2012,32 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.294</v>
+        <v>0.394</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>□60×60×3 (обрезки заказчика)</t>
+          <t>□100×60×4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>обрезок 2.80 м</t>
+          <t>1 (12 м)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2.403</t>
+          <t>4.013 + 3.993 + 3.833</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы — из обрезка заказчика</t>
+          <t>Колонна Л3; Колонна П1; Колонна П3</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.394</v>
+        <v>0.152</v>
       </c>
     </row>
     <row r="6">
@@ -2013,46 +2048,46 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1 (12 м)</t>
+          <t>2 (12 м)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4.013 + 3.993 + 3.833</t>
+          <t>3.803</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Колонна Л3; Колонна П1; Колонна П3</t>
+          <t>Колонна Л1</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.152</v>
+        <v>8.194000000000001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>□100×60×4</t>
+          <t>□100×60×3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2 (12 м)</t>
+          <t>1 (12 м)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>3.803</t>
+          <t>3.710 + 3.710 + 3.710</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Колонна Л1</t>
+          <t>Стропило длинное (свес 0.90)</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>8.194000000000001</v>
+        <v>0.861</v>
       </c>
     </row>
     <row r="8">
@@ -2063,46 +2098,46 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1 (12 м)</t>
+          <t>2 (12 м)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3.710 + 3.710 + 3.710</t>
+          <t>3.199 + 3.199 + 3.199</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Стропило длинное (свес 0.90)</t>
+          <t>Стропило короткое (свес 0.40)</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.861</v>
+        <v>2.394</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>□100×60×3</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2 (12 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>3.199 + 3.199 + 3.199</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Стропило короткое (свес 0.40)</t>
+          <t>Коньковая обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>2.394</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="10">
@@ -2113,21 +2148,21 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>5.397</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Коньковая обрешётина, часть 1 (передний край → стык)</t>
+          <t>Затяжка средней рамы</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.507</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="11">
@@ -2138,21 +2173,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>5.397</t>
+          <t>5.357</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Затяжка средней рамы</t>
+          <t>Затяжка крайней рамы</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.6</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="12">
@@ -2163,7 +2198,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>3 (6 м)</t>
+          <t>4 (6 м)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2188,21 +2223,21 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>4 (6 м)</t>
+          <t>5 (6 м)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>5.357</t>
+          <t>4.540</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Затяжка крайней рамы</t>
+          <t>Нижний пояс боковой фермы</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.64</v>
+        <v>1.457</v>
       </c>
     </row>
     <row r="14">
@@ -2213,7 +2248,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>5 (6 м)</t>
+          <t>6 (6 м)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2238,46 +2273,46 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>6 (6 м)</t>
+          <t>7 (6 м)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>4.540</t>
+          <t>2.403 + 2.403</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы</t>
+          <t>Раскос боковой фермы</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>1.457</v>
+        <v>1.188</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□30×30×2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>7 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2.403 + 2.403</t>
+          <t>0.598 + 0.598 + 0.598 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы</t>
+          <t>Вкладыш стыка обрешётины; Подвеска у конька</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1.188</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="17">
@@ -2308,51 +2343,51 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>□20×20×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.598 + 0.598 + 0.598</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Подвеска у конька</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>4.197</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>□30×30×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Вкладыш стыка обрешётины</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>4.043</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="20">
@@ -2363,7 +2398,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2388,7 +2423,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>4 (6 м)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2413,7 +2448,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>3 (6 м)</t>
+          <t>5 (6 м)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2438,7 +2473,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>4 (6 м)</t>
+          <t>6 (6 м)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2463,7 +2498,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>5 (6 м)</t>
+          <t>7 (6 м)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2488,7 +2523,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>6 (6 м)</t>
+          <t>8 (6 м)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2513,7 +2548,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>7 (6 м)</t>
+          <t>9 (6 м)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2538,7 +2573,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>8 (6 м)</t>
+          <t>10 (6 м)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2563,7 +2598,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>9 (6 м)</t>
+          <t>11 (6 м)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2588,7 +2623,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10 (6 м)</t>
+          <t>12 (6 м)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2613,7 +2648,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>11 (6 м)</t>
+          <t>13 (6 м)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2638,7 +2673,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>12 (6 м)</t>
+          <t>14 (6 м)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2663,7 +2698,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>13 (6 м)</t>
+          <t>15 (6 м)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2688,7 +2723,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>14 (6 м)</t>
+          <t>16 (6 м)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2713,7 +2748,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>15 (6 м)</t>
+          <t>17 (6 м)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2738,7 +2773,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>16 (6 м)</t>
+          <t>18 (6 м)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2763,7 +2798,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>17 (6 м)</t>
+          <t>19 (6 м)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2788,21 +2823,21 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>18 (6 м)</t>
+          <t>20 (6 м)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.507</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="38">
@@ -2813,21 +2848,21 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>19 (6 м)</t>
+          <t>21 (6 м)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.507</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="39">
@@ -2838,7 +2873,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>20 (6 м)</t>
+          <t>22 (6 м)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2863,7 +2898,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>21 (6 м)</t>
+          <t>23 (6 м)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2888,12 +2923,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>22 (6 м)</t>
+          <t>24 (6 м)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+          <t>1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2902,57 +2937,57 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0.028</v>
+        <v>1.521</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>23 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.028</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>24 (6 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>1.521</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="44">
@@ -2963,21 +2998,21 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>3.698 + 1.490</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
+          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край); Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.507</v>
+        <v>0.806</v>
       </c>
     </row>
     <row r="45">
@@ -2988,21 +3023,21 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>4 (6 м)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>3.698 + 1.490</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
+          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край); Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.507</v>
+        <v>0.806</v>
       </c>
     </row>
     <row r="46">
@@ -3013,21 +3048,21 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>3 (6 м)</t>
+          <t>5 (6 м)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>3.698 + 1.490</t>
+          <t>3.186</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край); Торцевая обвязка (по скату, под обрешёткой)</t>
+          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.806</v>
+        <v>2.811</v>
       </c>
     </row>
     <row r="47">
@@ -3038,70 +3073,20 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>4 (6 м)</t>
+          <t>6 (6 м)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>3.698 + 1.490</t>
+          <t>3.186</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край); Торцевая обвязка (по скату, под обрешёткой)</t>
+          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0.806</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>□50×30×2</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>5 (6 м)</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>3.186</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
-        </is>
-      </c>
-      <c r="E48" t="n">
-        <v>2.811</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>□50×30×2</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>6 (6 м)</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>3.186</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
-        </is>
-      </c>
-      <c r="E49" t="n">
         <v>2.811</v>
       </c>
     </row>
@@ -3919,13 +3904,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>24.29</v>
+        <v>24.3</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>2.481</v>
+        <v>2.484</v>
       </c>
       <c r="F2" t="n">
         <v>0.853</v>
@@ -3948,13 +3933,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>27.82</v>
+        <v>27.83</v>
       </c>
       <c r="D3" t="n">
         <v>1.09</v>
       </c>
       <c r="E3" t="n">
-        <v>4.078</v>
+        <v>4.076</v>
       </c>
       <c r="F3" t="n">
         <v>0.958</v>
@@ -3980,10 +3965,10 @@
         <v>0.31</v>
       </c>
       <c r="D4" t="n">
-        <v>26.26</v>
+        <v>26.27</v>
       </c>
       <c r="E4" t="n">
-        <v>0.37</v>
+        <v>0.374</v>
       </c>
       <c r="F4" t="n">
         <v>0.772</v>
@@ -4002,24 +3987,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>□20×20×2</t>
+          <t>□30×30×2</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>1.66</v>
+        <v>1.68</v>
       </c>
       <c r="E5" t="n">
-        <v>0.018</v>
+        <v>0.044</v>
       </c>
       <c r="F5" t="n">
-        <v>0.306</v>
+        <v>0.286</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>узел kp→tie: продавливание грани пояса N=1.7 кН, NRd=5.4 кН</t>
+          <t>стенка c/t изг. [D+S]</t>
         </is>
       </c>
     </row>
@@ -4035,13 +4020,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5.42</v>
+        <v>5.43</v>
       </c>
       <c r="D6" t="n">
-        <v>2.87</v>
+        <v>2.85</v>
       </c>
       <c r="E6" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.008</v>
       </c>
       <c r="F6" t="n">
         <v>0.889</v>
@@ -4064,16 +4049,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.75</v>
+        <v>1.76</v>
       </c>
       <c r="D7" t="n">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="E7" t="n">
         <v>0.453</v>
       </c>
       <c r="F7" t="n">
-        <v>0.949</v>
+        <v>0.948</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -4096,13 +4081,13 @@
         <v>1.3</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="E8" t="n">
         <v>0.258</v>
       </c>
       <c r="F8" t="n">
-        <v>0.655</v>
+        <v>0.656</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -4154,10 +4139,10 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>3.08</v>
+        <v>3.09</v>
       </c>
       <c r="E10" t="n">
-        <v>0.912</v>
+        <v>0.916</v>
       </c>
       <c r="F10" t="n">
         <v>0.643</v>
@@ -4180,7 +4165,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>21.02</v>
+        <v>21.03</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -4244,10 +4229,10 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>1.991</v>
+        <v>1.995</v>
       </c>
       <c r="F13" t="n">
-        <v>0.847</v>
+        <v>0.849</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Hanger back to 20×20×2; lath splice inserts removed (butt weld on a flat shelf), no 30×30 profile
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X6AG5Fdm1RBCCrsAG1aTU6
</commit_message>
<xml_diff>
--- a/output/smeta_optimized.xlsx
+++ b/output/smeta_optimized.xlsx
@@ -480,7 +480,7 @@
         <v>75812</v>
       </c>
       <c r="C2" t="n">
-        <v>47178</v>
+        <v>47095</v>
       </c>
       <c r="D2">
         <f>C2-B2</f>
@@ -678,7 +678,7 @@
         <v>5500</v>
       </c>
       <c r="C11" t="n">
-        <v>4213</v>
+        <v>4206</v>
       </c>
       <c r="D11">
         <f>C11-B11</f>
@@ -700,7 +700,7 @@
         <v>6600</v>
       </c>
       <c r="C12" t="n">
-        <v>5277</v>
+        <v>5235</v>
       </c>
       <c r="D12">
         <f>C12-B12</f>
@@ -810,7 +810,7 @@
         <v>24000</v>
       </c>
       <c r="C17" t="n">
-        <v>20153</v>
+        <v>20096</v>
       </c>
       <c r="D17">
         <f>C17-B17</f>
@@ -832,7 +832,7 @@
         <v>7000</v>
       </c>
       <c r="C18" t="n">
-        <v>5362</v>
+        <v>5353</v>
       </c>
       <c r="D18">
         <f>C18-B18</f>
@@ -854,7 +854,7 @@
         <v>15000</v>
       </c>
       <c r="C19" t="n">
-        <v>12596</v>
+        <v>12560</v>
       </c>
       <c r="D19">
         <f>C19-B19</f>
@@ -920,7 +920,7 @@
         <v>7000</v>
       </c>
       <c r="C22" t="n">
-        <v>5878</v>
+        <v>5861</v>
       </c>
       <c r="D22">
         <f>C22-B22</f>
@@ -961,7 +961,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Масса металла: было 1226 кг, стало 812 кг; площадь окраски 57.6 → 44.1 м²; швы 37.6 → 30.0 м; деталей 84 → 78.</t>
+          <t>Масса металла: было 1226 кг, стало 810 кг; площадь окраски 57.6 → 44.0 м²; швы 37.6 → 29.8 м; деталей 84 → 78.</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1168,73 +1168,46 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Подкосы фермы</t>
+          <t>Подвеска (стойка у конька), Подкосы фермы</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6.65</v>
+        <v>8.69</v>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>7</v>
+        <v>9.1</v>
       </c>
       <c r="F7" t="n">
         <v>67.40000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>448</v>
+        <v>586</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>□30×30×2</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Подвеска (стойка у конька)</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="D8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E8" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="F8" t="n">
-        <v>108</v>
-      </c>
-      <c r="G8" t="n">
-        <v>221</v>
+          <t>ИТОГО трубы</t>
+        </is>
+      </c>
+      <c r="C8">
+        <f>SUM(C2:C7)</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>SUM(E2:E7)</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>SUM(G2:G7)</f>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
-        <is>
-          <t>ИТОГО трубы</t>
-        </is>
-      </c>
-      <c r="C9">
-        <f>SUM(C2:C8)</f>
-        <v/>
-      </c>
-      <c r="E9">
-        <f>SUM(E2:E8)</f>
-        <v/>
-      </c>
-      <c r="G9">
-        <f>SUM(G2:G8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
         <is>
           <t>Пластины (фасонки, крышки колонн): 30.1 кг × 55 грн/кг</t>
         </is>
@@ -1251,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1510,7 +1483,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>□30×30×2</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1520,7 +1493,7 @@
         <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>1.9</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1557,33 +1530,33 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Вкладыш стыка обрешётины</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>□30×30×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.1</v>
+        <v>5.49</v>
       </c>
       <c r="D12" t="n">
         <v>19</v>
       </c>
       <c r="E12" t="n">
-        <v>3.2</v>
+        <v>207.7</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>отрезок трубы внутрь стыка, по 50 мм в каждую часть (по желанию)</t>
+          <t>торцы прямые; стык с частью 2 — в пролёте, в 290 мм от стропила рамы 3 (встык, см. узлы)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1592,43 +1565,43 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5.49</v>
+        <v>1.49</v>
       </c>
       <c r="D13" t="n">
         <v>19</v>
       </c>
       <c r="E13" t="n">
-        <v>207.7</v>
+        <v>56.4</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>торцы прямые; стык с частью 2 — в пролёте, в 290 мм от стропила рамы 3 (на вкладыше, см. узлы)</t>
+          <t>торцы прямые</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1.49</v>
+        <v>3.698</v>
       </c>
       <c r="D14" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>56.4</v>
+        <v>17.1</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>торцы прямые</t>
+          <t>у карниза — прямой рез, у конька — вертикальный рез (78° к оси) встык со второй половиной</t>
         </is>
       </c>
     </row>
@@ -1644,13 +1617,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3.698</v>
+        <v>3.186</v>
       </c>
       <c r="D15" t="n">
         <v>2</v>
       </c>
       <c r="E15" t="n">
-        <v>17.1</v>
+        <v>14.7</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1661,7 +1634,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
+          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1670,24 +1643,24 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3.186</v>
+        <v>5.49</v>
       </c>
       <c r="D16" t="n">
         <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>14.7</v>
+        <v>25.3</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>у карниза — прямой рез, у конька — вертикальный рез (78° к оси) встык со второй половиной</t>
+          <t>торцы прямые; стык с частью 2 — в пролёте, в 290 мм от стропила рамы 3 (встык, см. узлы)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
+          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1696,107 +1669,107 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>5.49</v>
+        <v>1.49</v>
       </c>
       <c r="D17" t="n">
         <v>2</v>
       </c>
       <c r="E17" t="n">
-        <v>25.3</v>
+        <v>6.9</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>торцы прямые; стык с частью 2 — в пролёте, в 290 мм от стропила рамы 3 (на вкладыше, см. узлы)</t>
+          <t>торцы прямые</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край)</t>
+          <t>Коньковая обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>□50×30×2</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1.49</v>
+        <v>5.49</v>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>6.9</v>
+        <v>19.6</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>торцы прямые</t>
+          <t>торцы прямые; стык с частью 2 — в пролёте, в 290 мм от стропила рамы 3 (встык, см. узлы)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Коньковая обрешётина, часть 1 (передний край → стык)</t>
+          <t>Коньковая обрешётина, часть 2 (стык → задний край) — из обрезка заказчика</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□60×60×3</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>5.49</v>
+        <v>1.49</v>
       </c>
       <c r="D19" t="n">
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>19.6</v>
+        <v>7.7</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>торцы прямые; стык с частью 2 — в пролёте, в 290 мм от стропила рамы 3 (на вкладыше, см. узлы)</t>
+          <t>торцы прямые; □60×60×3 вместо □60×60×2 — размеры и резы те же</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Коньковая обрешётина, часть 2 (стык → задний край) — из обрезка заказчика</t>
+          <t>Раскос боковой фермы</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>□60×60×3</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1.49</v>
+        <v>2.403</v>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20" t="n">
-        <v>7.7</v>
+        <v>17.1</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>торцы прямые; □60×60×3 вместо □60×60×2 — размеры и резы те же</t>
+          <t>оба торца — горизонтальные резы под 20.7° к оси (рез по грани 170 мм): низ — на пояс, верх — под столик</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы</t>
+          <t>Раскос боковой фермы — из обрезка заказчика</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□60×60×3</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1806,87 +1779,61 @@
         <v>2</v>
       </c>
       <c r="E21" t="n">
-        <v>17.1</v>
+        <v>24.9</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>оба торца — горизонтальные резы под 20.7° к оси (рез по грани 170 мм): низ — на пояс, верх — под столик</t>
+          <t>оба торца — горизонтальные резы под 20.7° к оси (рез по грани 170 мм): низ — на пояс, верх — под столик; □60×60×3 вместо □60×60×2 — размеры и резы те же</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы — из обрезка заказчика</t>
+          <t>Нижний пояс боковой фермы</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>□60×60×3</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2.403</v>
+        <v>4.54</v>
       </c>
       <c r="D22" t="n">
         <v>2</v>
       </c>
       <c r="E22" t="n">
-        <v>24.9</v>
+        <v>32.3</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>оба торца — горизонтальные резы под 20.7° к оси (рез по грани 170 мм): низ — на пояс, верх — под столик; □60×60×3 вместо □60×60×2 — размеры и резы те же</t>
+          <t>оба торца — прямые; по фактическому расстоянию между гранями колонн</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы</t>
+          <t>Стойка-вставка — из обрезка заказчика</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□60×60×3</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4.54</v>
+        <v>0.113</v>
       </c>
       <c r="D23" t="n">
         <v>2</v>
       </c>
       <c r="E23" t="n">
-        <v>32.3</v>
+        <v>1.2</v>
       </c>
       <c r="F23" t="inlineStr">
-        <is>
-          <t>оба торца — прямые; по фактическому расстоянию между гранями колонн</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Стойка-вставка — из обрезка заказчика</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>□60×60×3</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>0.113</v>
-      </c>
-      <c r="D24" t="n">
-        <v>2</v>
-      </c>
-      <c r="E24" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="F24" t="inlineStr">
         <is>
           <t>низ — прямой (встаёт на столик фермы), верх — под 12°</t>
         </is>
@@ -2293,7 +2240,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>□30×30×2</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2303,16 +2250,16 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.598 + 0.598 + 0.598 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100 + 0.100</t>
+          <t>0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.950</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Вкладыш стыка обрешётины; Подвеска у конька</t>
+          <t>Подкос фермы</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>2.24</v>
+        <v>0.282</v>
       </c>
     </row>
     <row r="17">
@@ -2323,21 +2270,21 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.950 + 0.950 + 0.950 + 0.950 + 0.950 + 0.950</t>
+          <t>0.598 + 0.598 + 0.598</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Подкос фермы</t>
+          <t>Подвеска у конька</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.282</v>
+        <v>4.197</v>
       </c>
     </row>
     <row r="18">
@@ -3904,13 +3851,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>24.3</v>
+        <v>24.29</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>2.484</v>
+        <v>2.481</v>
       </c>
       <c r="F2" t="n">
         <v>0.853</v>
@@ -3933,13 +3880,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>27.83</v>
+        <v>27.82</v>
       </c>
       <c r="D3" t="n">
         <v>1.09</v>
       </c>
       <c r="E3" t="n">
-        <v>4.076</v>
+        <v>4.078</v>
       </c>
       <c r="F3" t="n">
         <v>0.958</v>
@@ -3965,10 +3912,10 @@
         <v>0.31</v>
       </c>
       <c r="D4" t="n">
-        <v>26.27</v>
+        <v>26.26</v>
       </c>
       <c r="E4" t="n">
-        <v>0.374</v>
+        <v>0.37</v>
       </c>
       <c r="F4" t="n">
         <v>0.772</v>
@@ -3987,24 +3934,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>□30×30×2</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>1.68</v>
+        <v>1.66</v>
       </c>
       <c r="E5" t="n">
-        <v>0.044</v>
+        <v>0.018</v>
       </c>
       <c r="F5" t="n">
-        <v>0.286</v>
+        <v>0.306</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>стенка c/t изг. [D+S]</t>
+          <t>узел kp→tie: продавливание грани пояса N=1.7 кН, NRd=5.4 кН</t>
         </is>
       </c>
     </row>
@@ -4020,13 +3967,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5.43</v>
+        <v>5.42</v>
       </c>
       <c r="D6" t="n">
-        <v>2.85</v>
+        <v>2.87</v>
       </c>
       <c r="E6" t="n">
-        <v>0.008</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="F6" t="n">
         <v>0.889</v>
@@ -4049,16 +3996,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.76</v>
+        <v>1.75</v>
       </c>
       <c r="D7" t="n">
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
       <c r="E7" t="n">
         <v>0.453</v>
       </c>
       <c r="F7" t="n">
-        <v>0.948</v>
+        <v>0.949</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -4081,13 +4028,13 @@
         <v>1.3</v>
       </c>
       <c r="D8" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="E8" t="n">
         <v>0.258</v>
       </c>
       <c r="F8" t="n">
-        <v>0.656</v>
+        <v>0.655</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -4139,10 +4086,10 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>3.09</v>
+        <v>3.08</v>
       </c>
       <c r="E10" t="n">
-        <v>0.916</v>
+        <v>0.912</v>
       </c>
       <c r="F10" t="n">
         <v>0.643</v>
@@ -4165,7 +4112,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>21.03</v>
+        <v>21.02</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -4229,10 +4176,10 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>1.995</v>
+        <v>1.991</v>
       </c>
       <c r="F13" t="n">
-        <v>0.849</v>
+        <v>0.847</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Ridge lath on rafter apex: Ø6 rods in the 6.4 mm wedge gap, weld 14; detail drawing, parts list and reply updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X6AG5Fdm1RBCCrsAG1aTU6
</commit_message>
<xml_diff>
--- a/output/smeta_optimized.xlsx
+++ b/output/smeta_optimized.xlsx
@@ -3445,7 +3445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3749,31 +3749,64 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Пруток Ø6 под коньковую обрешётину</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Ø6: 6 × 60 + 4 × 30 мм</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>клиновой зазор под коньковой обрешётиной на стропилах (6) и на обвязке (4)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>катанка / арматура Ø6, ≈ 0.5 м</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Заглушка торца коньковой обрешётины</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>60 × 60</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D11" t="n">
         <v>2</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E11" t="n">
         <v>0</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>торцы коньковой обрешётины</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>пластиковые заглушки 60×60</t>
         </is>

</xml_diff>

<commit_message>
Columns concreted full hole depth (bottom 10 cm above hole bottom), no hole rebar; lengths, cutting, estimate, assembly steps and reply updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X6AG5Fdm1RBCCrsAG1aTU6
</commit_message>
<xml_diff>
--- a/output/smeta_optimized.xlsx
+++ b/output/smeta_optimized.xlsx
@@ -480,7 +480,7 @@
         <v>75812</v>
       </c>
       <c r="C2" t="n">
-        <v>47095</v>
+        <v>48094</v>
       </c>
       <c r="D2">
         <f>C2-B2</f>
@@ -524,7 +524,7 @@
         <v>3000</v>
       </c>
       <c r="C4" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="D4">
         <f>C4-B4</f>
@@ -678,7 +678,7 @@
         <v>5500</v>
       </c>
       <c r="C11" t="n">
-        <v>4206</v>
+        <v>4233</v>
       </c>
       <c r="D11">
         <f>C11-B11</f>
@@ -810,7 +810,7 @@
         <v>24000</v>
       </c>
       <c r="C17" t="n">
-        <v>20096</v>
+        <v>20116</v>
       </c>
       <c r="D17">
         <f>C17-B17</f>
@@ -832,7 +832,7 @@
         <v>7000</v>
       </c>
       <c r="C18" t="n">
-        <v>5353</v>
+        <v>5387</v>
       </c>
       <c r="D18">
         <f>C18-B18</f>
@@ -854,7 +854,7 @@
         <v>15000</v>
       </c>
       <c r="C19" t="n">
-        <v>12560</v>
+        <v>12572</v>
       </c>
       <c r="D19">
         <f>C19-B19</f>
@@ -920,7 +920,7 @@
         <v>7000</v>
       </c>
       <c r="C22" t="n">
-        <v>5861</v>
+        <v>5867</v>
       </c>
       <c r="D22">
         <f>C22-B22</f>
@@ -961,7 +961,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Масса металла: было 1226 кг, стало 810 кг; площадь окраски 57.6 → 44.0 м²; швы 37.6 → 29.8 м; деталей 84 → 78.</t>
+          <t>Масса металла: было 1226 кг, стало 828 кг; площадь окраски 57.6 → 44.3 м²; швы 37.6 → 29.8 м; деталей 84 → 78.</t>
         </is>
       </c>
     </row>
@@ -1055,55 +1055,55 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>□100×60×3</t>
+          <t>□100×60×4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Стропила</t>
+          <t>Колонны</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20.75</v>
+        <v>17.5</v>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>146.7</v>
+        <v>161.4</v>
       </c>
       <c r="F3" t="n">
-        <v>428</v>
+        <v>540</v>
       </c>
       <c r="G3" t="n">
-        <v>8879</v>
+        <v>9452</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>□100×60×4</t>
+          <t>□100×60×3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Колонны</t>
+          <t>Стропила</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>15.65</v>
+        <v>20.75</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E4" t="n">
-        <v>144.4</v>
+        <v>146.7</v>
       </c>
       <c r="F4" t="n">
-        <v>540</v>
+        <v>428</v>
       </c>
       <c r="G4" t="n">
-        <v>8453</v>
+        <v>8879</v>
       </c>
     </row>
     <row r="5">
@@ -1279,17 +1279,17 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3.803</v>
+        <v>4.203</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>35.1</v>
+        <v>38.8</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>низ — прямой рез (+ заглушка), верх — под 12° по низу стропила; в бетоне 0.70 м</t>
+          <t>низ — прямой рез (+ заглушка), верх — под 12° по низу стропила; в бетоне 1.10 м (на всю глубину лунки, низ на 10 см выше дна)</t>
         </is>
       </c>
     </row>
@@ -1305,17 +1305,17 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3.993</v>
+        <v>4.393</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>36.8</v>
+        <v>40.5</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>низ — прямой рез (+ заглушка), верх — под 12° по низу стропила; в бетоне 0.70 м</t>
+          <t>низ — прямой рез (+ заглушка), верх — под 12° по низу стропила; в бетоне 1.10 м (на всю глубину лунки, низ на 10 см выше дна)</t>
         </is>
       </c>
     </row>
@@ -1331,17 +1331,17 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3.833</v>
+        <v>4.333</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>35.3</v>
+        <v>40</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>низ — прямой рез (+ заглушка), верх — под 12° по низу стропила; в бетоне 0.70 м</t>
+          <t>низ — прямой рез (+ заглушка), верх — под 12° по низу стропила; в бетоне 1.20 м (на всю глубину лунки, низ на 10 см выше дна)</t>
         </is>
       </c>
     </row>
@@ -1357,17 +1357,17 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4.013</v>
+        <v>4.563</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>37</v>
+        <v>42.1</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>низ — прямой рез (+ заглушка), верх — под 12° по низу стропила; в бетоне 0.70 м</t>
+          <t>низ — прямой рез (+ заглушка), верх — под 12° по низу стропила; в бетоне 1.25 м (на всю глубину лунки, низ на 10 см выше дна)</t>
         </is>
       </c>
     </row>
@@ -1975,16 +1975,16 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4.013 + 3.993 + 3.833</t>
+          <t>4.563 + 4.393</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Колонна Л3; Колонна П1; Колонна П3</t>
+          <t>Колонна Л3; Колонна П3</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.152</v>
+        <v>3.038</v>
       </c>
     </row>
     <row r="6">
@@ -2000,16 +2000,16 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3.803</t>
+          <t>4.333 + 4.203</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Колонна Л1</t>
+          <t>Колонна Л1; Колонна П1</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>8.194000000000001</v>
+        <v>3.458</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Roof document (krovlya.html/pdf): tile layout and flat 200x200 ridge cap (section, spec, mounting); sheet gap at ridge 50 mm so sheets clear the 60x60 ridge lath
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X6AG5Fdm1RBCCrsAG1aTU6
</commit_message>
<xml_diff>
--- a/output/smeta_optimized.xlsx
+++ b/output/smeta_optimized.xlsx
@@ -3101,17 +3101,17 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>3.21</v>
+        <v>3.19</v>
       </c>
       <c r="D2" t="n">
         <v>1100</v>
       </c>
       <c r="E2" t="n">
-        <v>943</v>
+        <v>944</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>передняя кромка 0→157 мм</t>
+          <t>передняя кромка 0→156 мм</t>
         </is>
       </c>
     </row>
@@ -3125,7 +3125,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>3.21</v>
+        <v>3.19</v>
       </c>
       <c r="D3" t="n">
         <v>1100</v>
@@ -3149,7 +3149,7 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>3.21</v>
+        <v>3.19</v>
       </c>
       <c r="D4" t="n">
         <v>1100</v>
@@ -3173,7 +3173,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>3.21</v>
+        <v>3.19</v>
       </c>
       <c r="D5" t="n">
         <v>1100</v>
@@ -3197,7 +3197,7 @@
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>3.21</v>
+        <v>3.19</v>
       </c>
       <c r="D6" t="n">
         <v>1100</v>
@@ -3221,7 +3221,7 @@
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>3.21</v>
+        <v>3.19</v>
       </c>
       <c r="D7" t="n">
         <v>1100</v>
@@ -3245,17 +3245,17 @@
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>3.21</v>
+        <v>3.19</v>
       </c>
       <c r="D8" t="n">
         <v>380</v>
       </c>
       <c r="E8" t="n">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>задняя кромка 720→562 мм</t>
+          <t>задняя кромка 720→563 мм</t>
         </is>
       </c>
     </row>
@@ -3269,17 +3269,17 @@
         <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>3.721</v>
+        <v>3.701</v>
       </c>
       <c r="D9" t="n">
-        <v>918</v>
+        <v>919</v>
       </c>
       <c r="E9" t="n">
         <v>1100</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>передняя кромка 182→0 мм</t>
+          <t>передняя кромка 181→0 мм</t>
         </is>
       </c>
     </row>
@@ -3293,7 +3293,7 @@
         <v>2</v>
       </c>
       <c r="C10" t="n">
-        <v>3.721</v>
+        <v>3.701</v>
       </c>
       <c r="D10" t="n">
         <v>1100</v>
@@ -3317,7 +3317,7 @@
         <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>3.721</v>
+        <v>3.701</v>
       </c>
       <c r="D11" t="n">
         <v>1100</v>
@@ -3341,7 +3341,7 @@
         <v>4</v>
       </c>
       <c r="C12" t="n">
-        <v>3.721</v>
+        <v>3.701</v>
       </c>
       <c r="D12" t="n">
         <v>1100</v>
@@ -3365,7 +3365,7 @@
         <v>5</v>
       </c>
       <c r="C13" t="n">
-        <v>3.721</v>
+        <v>3.701</v>
       </c>
       <c r="D13" t="n">
         <v>1100</v>
@@ -3389,7 +3389,7 @@
         <v>6</v>
       </c>
       <c r="C14" t="n">
-        <v>3.721</v>
+        <v>3.701</v>
       </c>
       <c r="D14" t="n">
         <v>1100</v>
@@ -3413,24 +3413,24 @@
         <v>7</v>
       </c>
       <c r="C15" t="n">
-        <v>3.721</v>
+        <v>3.701</v>
       </c>
       <c r="D15" t="n">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="E15" t="n">
         <v>380</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>задняя кромка 537→720 мм</t>
+          <t>задняя кромка 538→720 мм</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Итого 14 листов; площадь по габаритной ширине 1.18 м — 57.2 м², по полезной — 53.4 м²; кровля 48.2 м². Укладка от переднего края (дорога).</t>
+          <t>Итого 14 листов; площадь по габаритной ширине 1.18 м — 56.9 м², по полезной — 53.1 м²; кровля 48.2 м². Укладка от переднего края (дорога).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adopted design: polycarbonate side panel on the right column row (cp 1.8) and 20x20x2 truss diagonals at the supports in all frames
Instead of reinforcing the right rafters, one extra diagonal per half-frame from the truss strut node on the
rafter down to the tie at 0.85 m from the column axis (6 pcs, same look in all frames). Frame maximum 0.935
(laths), rafters 0.88 (without the diagonals 1.09). Top panel rail is split at the middle-frame stub (two simple
spans welded to the A and B gussets), panel load distribution updated. Report compares the scheme search with the
adopted design without the panel; montage order in uzly gets the diagonals step (seam 15).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MjM9cRLPNnoPi19GB3uSre
</commit_message>
<xml_diff>
--- a/output/smeta_optimized.xlsx
+++ b/output/smeta_optimized.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Сравнение" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Ведомость металла" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Детали" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Раскрой на хлысты" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Металлочерепица" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Пластины" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Проверки" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Варианты схем" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Нагрузки" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сравнение" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ведомость металла" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Детали" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Раскрой на хлысты" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Металлочерепица" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Пластины" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Проверки" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Варианты схем" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нагрузки" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -480,7 +480,7 @@
         <v>75812</v>
       </c>
       <c r="C2" t="n">
-        <v>48094</v>
+        <v>48497</v>
       </c>
       <c r="D2">
         <f>C2-B2</f>
@@ -678,7 +678,7 @@
         <v>5500</v>
       </c>
       <c r="C11" t="n">
-        <v>4233</v>
+        <v>4274</v>
       </c>
       <c r="D11">
         <f>C11-B11</f>
@@ -700,7 +700,7 @@
         <v>6600</v>
       </c>
       <c r="C12" t="n">
-        <v>5235</v>
+        <v>5389</v>
       </c>
       <c r="D12">
         <f>C12-B12</f>
@@ -810,7 +810,7 @@
         <v>24000</v>
       </c>
       <c r="C17" t="n">
-        <v>20116</v>
+        <v>21500</v>
       </c>
       <c r="D17">
         <f>C17-B17</f>
@@ -832,7 +832,7 @@
         <v>7000</v>
       </c>
       <c r="C18" t="n">
-        <v>5387</v>
+        <v>5440</v>
       </c>
       <c r="D18">
         <f>C18-B18</f>
@@ -854,7 +854,7 @@
         <v>15000</v>
       </c>
       <c r="C19" t="n">
-        <v>12572</v>
+        <v>13437</v>
       </c>
       <c r="D19">
         <f>C19-B19</f>
@@ -920,7 +920,7 @@
         <v>7000</v>
       </c>
       <c r="C22" t="n">
-        <v>5867</v>
+        <v>6271</v>
       </c>
       <c r="D22">
         <f>C22-B22</f>
@@ -961,7 +961,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Масса металла: было 1226 кг, стало 828 кг; площадь окраски 57.6 → 44.3 м²; швы 37.6 → 29.8 м; деталей 84 → 78.</t>
+          <t>Масса металла: было 1226 кг, стало 834 кг; площадь окраски 57.6 → 44.7 м²; швы 37.6 → 30.7 м; деталей 84 → 84.</t>
         </is>
       </c>
     </row>
@@ -1168,23 +1168,23 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Подвеска (стойка у конька), Подкосы фермы</t>
+          <t>Доп. решётка ферм у опор, Подвеска (стойка у конька), Подкосы фермы</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>8.69</v>
+        <v>14.67</v>
       </c>
       <c r="D7" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E7" t="n">
-        <v>9.1</v>
+        <v>15.4</v>
       </c>
       <c r="F7" t="n">
         <v>67.40000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>586</v>
+        <v>989</v>
       </c>
     </row>
     <row r="8">
@@ -1224,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1530,33 +1530,33 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Раскос фермы у опоры</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>5.49</v>
+        <v>0.747</v>
       </c>
       <c r="D12" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="E12" t="n">
-        <v>207.7</v>
+        <v>4.7</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>торцы прямые; стык с частью 2 — в пролёте, в 290 мм от стропила рамы 3 (встык, см. узлы)</t>
+          <t>низ — под 28° к оси (на затяжку в 0.85 м от оси колонны), верх — под 16° (на стропило в узле подкоса)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1565,43 +1565,43 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1.49</v>
+        <v>5.49</v>
       </c>
       <c r="D13" t="n">
         <v>19</v>
       </c>
       <c r="E13" t="n">
-        <v>56.4</v>
+        <v>207.7</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>торцы прямые</t>
+          <t>торцы прямые; стык с частью 2 — в пролёте, в 290 мм от стропила рамы 3 (встык, см. узлы)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>□50×30×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3.698</v>
+        <v>1.49</v>
       </c>
       <c r="D14" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E14" t="n">
-        <v>17.1</v>
+        <v>56.4</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>у карниза — прямой рез, у конька — вертикальный рез (78° к оси) встык со второй половиной</t>
+          <t>торцы прямые</t>
         </is>
       </c>
     </row>
@@ -1617,13 +1617,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3.186</v>
+        <v>3.698</v>
       </c>
       <c r="D15" t="n">
         <v>2</v>
       </c>
       <c r="E15" t="n">
-        <v>14.7</v>
+        <v>17.1</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1634,7 +1634,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
+          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1643,24 +1643,24 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>5.49</v>
+        <v>3.186</v>
       </c>
       <c r="D16" t="n">
         <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>25.3</v>
+        <v>14.7</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>торцы прямые; стык с частью 2 — в пролёте, в 290 мм от стропила рамы 3 (встык, см. узлы)</t>
+          <t>у карниза — прямой рез, у конька — вертикальный рез (78° к оси) встык со второй половиной</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край)</t>
+          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1669,107 +1669,107 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.49</v>
+        <v>5.49</v>
       </c>
       <c r="D17" t="n">
         <v>2</v>
       </c>
       <c r="E17" t="n">
-        <v>6.9</v>
+        <v>25.3</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>торцы прямые</t>
+          <t>торцы прямые; стык с частью 2 — в пролёте, в 290 мм от стропила рамы 3 (встык, см. узлы)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Коньковая обрешётина, часть 1 (передний край → стык)</t>
+          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>5.49</v>
+        <v>1.49</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18" t="n">
-        <v>19.6</v>
+        <v>6.9</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>торцы прямые; стык с частью 2 — в пролёте, в 290 мм от стропила рамы 3 (встык, см. узлы)</t>
+          <t>торцы прямые</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Коньковая обрешётина, часть 2 (стык → задний край) — из обрезка заказчика</t>
+          <t>Коньковая обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>□60×60×3</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.49</v>
+        <v>5.49</v>
       </c>
       <c r="D19" t="n">
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>7.7</v>
+        <v>19.6</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>торцы прямые; □60×60×3 вместо □60×60×2 — размеры и резы те же</t>
+          <t>торцы прямые; стык с частью 2 — в пролёте, в 290 мм от стропила рамы 3 (встык, см. узлы)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы</t>
+          <t>Коньковая обрешётина, часть 2 (стык → задний край) — из обрезка заказчика</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□60×60×3</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2.403</v>
+        <v>1.49</v>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>17.1</v>
+        <v>7.7</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>оба торца — горизонтальные резы под 20.7° к оси (рез по грани 170 мм): низ — на пояс, верх — под столик</t>
+          <t>торцы прямые; □60×60×3 вместо □60×60×2 — размеры и резы те же</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Раскос боковой фермы — из обрезка заказчика</t>
+          <t>Раскос боковой фермы</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>□60×60×3</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1779,61 +1779,87 @@
         <v>2</v>
       </c>
       <c r="E21" t="n">
-        <v>24.9</v>
+        <v>17.1</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>оба торца — горизонтальные резы под 20.7° к оси (рез по грани 170 мм): низ — на пояс, верх — под столик; □60×60×3 вместо □60×60×2 — размеры и резы те же</t>
+          <t>оба торца — горизонтальные резы под 20.7° к оси (рез по грани 170 мм): низ — на пояс, верх — под столик</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы</t>
+          <t>Раскос боковой фермы — из обрезка заказчика</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□60×60×3</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4.54</v>
+        <v>2.403</v>
       </c>
       <c r="D22" t="n">
         <v>2</v>
       </c>
       <c r="E22" t="n">
-        <v>32.3</v>
+        <v>24.9</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>оба торца — прямые; по фактическому расстоянию между гранями колонн</t>
+          <t>оба торца — горизонтальные резы под 20.7° к оси (рез по грани 170 мм): низ — на пояс, верх — под столик; □60×60×3 вместо □60×60×2 — размеры и резы те же</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Стойка-вставка — из обрезка заказчика</t>
+          <t>Нижний пояс боковой фермы</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>□60×60×3</t>
+          <t>□60×60×2</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.113</v>
+        <v>4.54</v>
       </c>
       <c r="D23" t="n">
         <v>2</v>
       </c>
       <c r="E23" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>оба торца — прямые; по фактическому расстоянию между гранями колонн</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Стойка-вставка — из обрезка заказчика</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>□60×60×3</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0.113</v>
+      </c>
+      <c r="D24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" t="n">
         <v>1.2</v>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>низ — прямой (встаёт на столик фермы), верх — под 12°</t>
         </is>
@@ -1850,7 +1876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2275,41 +2301,41 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.598 + 0.598 + 0.598</t>
+          <t>0.747 + 0.747 + 0.747 + 0.747 + 0.747 + 0.747 + 0.598 + 0.598</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Подвеска у конька</t>
+          <t>Подвеска у конька; Раскос фермы у опоры</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>4.197</v>
+        <v>0.298</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>0.598</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 1 (передний край → стык)</t>
+          <t>Подвеска у конька</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.507</v>
+        <v>5.399</v>
       </c>
     </row>
     <row r="19">
@@ -2320,7 +2346,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2345,7 +2371,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>3 (6 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2370,7 +2396,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>4 (6 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2395,7 +2421,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>5 (6 м)</t>
+          <t>4 (6 м)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2420,7 +2446,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>6 (6 м)</t>
+          <t>5 (6 м)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2445,7 +2471,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>7 (6 м)</t>
+          <t>6 (6 м)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2470,7 +2496,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>8 (6 м)</t>
+          <t>7 (6 м)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2495,7 +2521,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>9 (6 м)</t>
+          <t>8 (6 м)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2520,7 +2546,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>10 (6 м)</t>
+          <t>9 (6 м)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2545,7 +2571,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>11 (6 м)</t>
+          <t>10 (6 м)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2570,7 +2596,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>12 (6 м)</t>
+          <t>11 (6 м)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2595,7 +2621,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>13 (6 м)</t>
+          <t>12 (6 м)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2620,7 +2646,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>14 (6 м)</t>
+          <t>13 (6 м)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2645,7 +2671,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>15 (6 м)</t>
+          <t>14 (6 м)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2670,7 +2696,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>16 (6 м)</t>
+          <t>15 (6 м)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2695,7 +2721,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>17 (6 м)</t>
+          <t>16 (6 м)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2720,7 +2746,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>18 (6 м)</t>
+          <t>17 (6 м)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2745,7 +2771,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>19 (6 м)</t>
+          <t>18 (6 м)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2770,21 +2796,21 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>20 (6 м)</t>
+          <t>19 (6 м)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490 + 1.490</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Обрешётина, часть 2 (стык → задний край)</t>
+          <t>Обрешётина, часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.028</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="38">
@@ -2795,7 +2821,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>21 (6 м)</t>
+          <t>20 (6 м)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2820,7 +2846,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>22 (6 м)</t>
+          <t>21 (6 м)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2845,7 +2871,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>23 (6 м)</t>
+          <t>22 (6 м)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2870,12 +2896,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>24 (6 м)</t>
+          <t>23 (6 м)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1.490 + 1.490 + 1.490</t>
+          <t>1.490 + 1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2884,32 +2910,32 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>1.521</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>□50×30×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1 (6 м)</t>
+          <t>24 (6 м)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>5.490</t>
+          <t>1.490 + 1.490 + 1.490</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
+          <t>Обрешётина, часть 2 (стык → задний край)</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.507</v>
+        <v>1.521</v>
       </c>
     </row>
     <row r="43">
@@ -2920,7 +2946,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2 (6 м)</t>
+          <t>1 (6 м)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2945,21 +2971,21 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>3 (6 м)</t>
+          <t>2 (6 м)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>3.698 + 1.490</t>
+          <t>5.490</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край); Торцевая обвязка (по скату, под обрешёткой)</t>
+          <t>Карнизная обрешётина (на ребро), часть 1 (передний край → стык)</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.806</v>
+        <v>0.507</v>
       </c>
     </row>
     <row r="45">
@@ -2970,7 +2996,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>4 (6 м)</t>
+          <t>3 (6 м)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2995,21 +3021,21 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>5 (6 м)</t>
+          <t>4 (6 м)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>3.186</t>
+          <t>3.698 + 1.490</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
+          <t>Карнизная обрешётина (на ребро), часть 2 (стык → задний край); Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>2.811</v>
+        <v>0.806</v>
       </c>
     </row>
     <row r="47">
@@ -3020,20 +3046,45 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t>5 (6 м)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>3.186</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Торцевая обвязка (по скату, под обрешёткой)</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>2.811</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>□50×30×2</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>6 (6 м)</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>3.186</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>Торцевая обвязка (по скату, под обрешёткой)</t>
         </is>
       </c>
-      <c r="E47" t="n">
+      <c r="E48" t="n">
         <v>2.811</v>
       </c>
     </row>
@@ -3823,7 +3874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3884,20 +3935,20 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>24.29</v>
+        <v>24.32</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>2.481</v>
+        <v>2.341</v>
       </c>
       <c r="F2" t="n">
-        <v>0.853</v>
+        <v>0.834</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>гибкость [D+S]</t>
+          <t>гибкость [D+S+0.9W+y]</t>
         </is>
       </c>
     </row>
@@ -3913,16 +3964,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>27.82</v>
+        <v>25.47</v>
       </c>
       <c r="D3" t="n">
-        <v>1.09</v>
+        <v>1.88</v>
       </c>
       <c r="E3" t="n">
-        <v>4.078</v>
+        <v>3.591</v>
       </c>
       <c r="F3" t="n">
-        <v>0.958</v>
+        <v>0.842</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -3942,20 +3993,20 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.31</v>
+        <v>2.36</v>
       </c>
       <c r="D4" t="n">
-        <v>26.26</v>
+        <v>26.1</v>
       </c>
       <c r="E4" t="n">
-        <v>0.37</v>
+        <v>1.186</v>
       </c>
       <c r="F4" t="n">
-        <v>0.772</v>
+        <v>0.789</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>гибкость [0.95D+W-x]</t>
+          <t>прочность [D+S+0.9W+x]</t>
         </is>
       </c>
     </row>
@@ -3971,20 +4022,20 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="D5" t="n">
-        <v>1.66</v>
+        <v>2.6</v>
       </c>
       <c r="E5" t="n">
         <v>0.018</v>
       </c>
       <c r="F5" t="n">
-        <v>0.306</v>
+        <v>0.526</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>узел kp→tie: продавливание грани пояса N=1.7 кН, NRd=5.4 кН</t>
+          <t>гибкость [0.95D+W-x]</t>
         </is>
       </c>
     </row>
@@ -4000,16 +4051,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5.42</v>
+        <v>5.54</v>
       </c>
       <c r="D6" t="n">
-        <v>2.87</v>
+        <v>2.85</v>
       </c>
       <c r="E6" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.005</v>
       </c>
       <c r="F6" t="n">
-        <v>0.889</v>
+        <v>0.893</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -4020,65 +4071,65 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Обрешётка</t>
+          <t>Доп. решётка ферм у опор</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>□35×35×2</t>
+          <t>□20×20×2</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1.75</v>
+        <v>4.47</v>
       </c>
       <c r="D7" t="n">
-        <v>0.85</v>
+        <v>1.08</v>
       </c>
       <c r="E7" t="n">
-        <v>0.453</v>
+        <v>0.02</v>
       </c>
       <c r="F7" t="n">
-        <v>0.949</v>
+        <v>0.769</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>устойчивость [D+S+0.9W-x]</t>
+          <t>гибкость [D+S+0.9W+x]</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Торцевая обвязка обрешётки</t>
+          <t>Обрешётка</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>□50×30×2</t>
+          <t>□35×35×2</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1.3</v>
+        <v>1.76</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1</v>
+        <v>0.87</v>
       </c>
       <c r="E8" t="n">
-        <v>0.258</v>
+        <v>0.446</v>
       </c>
       <c r="F8" t="n">
-        <v>0.655</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>устойчивость [D+S]</t>
+          <t>устойчивость [D+S+0.9W-x]</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Карнизные обрешётины</t>
+          <t>Торцевая обвязка обрешётки</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4087,56 +4138,56 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.6</v>
+        <v>1.29</v>
       </c>
       <c r="D9" t="n">
-        <v>0.06</v>
+        <v>0.11</v>
       </c>
       <c r="E9" t="n">
-        <v>0.51</v>
+        <v>0.262</v>
       </c>
       <c r="F9" t="n">
-        <v>0.734</v>
+        <v>0.659</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>устойчивость [D+S+0.9W+x]</t>
+          <t>устойчивость [D+S]</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Коньковая обрешётина</t>
+          <t>Карнизные обрешётины</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>□60×60×2</t>
+          <t>□50×30×2</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="D10" t="n">
-        <v>3.08</v>
+        <v>0.12</v>
       </c>
       <c r="E10" t="n">
-        <v>0.912</v>
+        <v>0.517</v>
       </c>
       <c r="F10" t="n">
-        <v>0.643</v>
+        <v>0.742</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>стенка c/t изг. [D+S]</t>
+          <t>устойчивость [D+S+0.9W+x]</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Раскосы боковой фермы</t>
+          <t>Коньковая обрешётина</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4145,27 +4196,27 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>21.02</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>3.09</v>
       </c>
       <c r="E11" t="n">
-        <v>0.181</v>
+        <v>0.914</v>
       </c>
       <c r="F11" t="n">
         <v>0.643</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>стенка c/t [D+S]</t>
+          <t>стенка c/t изг. [D+S]</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Нижний пояс боковой фермы</t>
+          <t>Раскосы боковой фермы</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4174,47 +4225,76 @@
         </is>
       </c>
       <c r="C12" t="n">
+        <v>21.04</v>
+      </c>
+      <c r="D12" t="n">
         <v>0</v>
       </c>
-      <c r="D12" t="n">
-        <v>18.01</v>
-      </c>
       <c r="E12" t="n">
-        <v>0.128</v>
+        <v>0.183</v>
       </c>
       <c r="F12" t="n">
         <v>0.643</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>стенка c/t изг. [D+S]</t>
+          <t>стенка c/t [D+S]</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Нижний пояс боковой фермы</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>□60×60×2</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>18.02</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.276</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.643</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>стенка c/t изг. [D+S]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Стойка-вставка средней рамы</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>□60×60×3</t>
         </is>
       </c>
-      <c r="C13" t="n">
+      <c r="C14" t="n">
         <v>14</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D14" t="n">
         <v>0</v>
       </c>
-      <c r="E13" t="n">
-        <v>1.991</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0.847</v>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="E14" t="n">
+        <v>1.511</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="G14" t="inlineStr">
         <is>
           <t>устойчивость [D+S]</t>
         </is>

</xml_diff>